<commit_message>
fix biosphere version in LCIs
</commit_message>
<xml_diff>
--- a/inventories/lci-lithium_brine_projects-optimized.xlsx
+++ b/inventories/lci-lithium_brine_projects-optimized.xlsx
@@ -31,7 +31,7 @@
     <t>code</t>
   </si>
   <si>
-    <t>2af6eefe41f04c79b9beda64628b2e60</t>
+    <t>95e06081ea49402b8b77dfbd02cccb9b</t>
   </si>
   <si>
     <t>location</t>
@@ -103,7 +103,7 @@
     <t>Water_Ang_Sal de los Angeles</t>
   </si>
   <si>
-    <t>e60a84e5fb7e4daaa32ab6ed6c54ce02</t>
+    <t>c9c945ccb7b24805af82f0cf472e11bc</t>
   </si>
   <si>
     <t>AR</t>
@@ -148,7 +148,7 @@
     <t>Water_Ari_Salar de Arizaro</t>
   </si>
   <si>
-    <t>4d5e163854c44f559c5233a462110a21</t>
+    <t>50c5511a9e56472ea84773419aa357b3</t>
   </si>
   <si>
     <t>Water_Ari</t>
@@ -169,7 +169,7 @@
     <t>Water_Ata_Salar de Atacama</t>
   </si>
   <si>
-    <t>e5c7faf0215648af94a2c02283e0880c</t>
+    <t>b00e44637bee4f92956034a432f249f3</t>
   </si>
   <si>
     <t>CL</t>
@@ -184,7 +184,7 @@
     <t>Water_Cau_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>c5a326e8f3514ccc870919d9f91f18c4</t>
+    <t>0a2db3ed162e4a929687bcefcdec5a7e</t>
   </si>
   <si>
     <t>Water_Cau</t>
@@ -196,7 +196,7 @@
     <t>Water_Cent_Salar de Centenario</t>
   </si>
   <si>
-    <t>cbdd60b459f2456d869b20b04fb62b4b</t>
+    <t>bef999cd3fc94936a7c8873184995b1b</t>
   </si>
   <si>
     <t>Water_Cent</t>
@@ -208,7 +208,7 @@
     <t>Water_Chaer_Chaerhan</t>
   </si>
   <si>
-    <t>5c67b405576e4fc192b85bbdb6573966</t>
+    <t>0058eb9d8b1848259728128b13a033aa</t>
   </si>
   <si>
     <t>CN-NWG</t>
@@ -223,7 +223,7 @@
     <t>Water_EaTai_East Taijinar</t>
   </si>
   <si>
-    <t>fa43bb44c31041628c9b4946591d89b0</t>
+    <t>c8d773f6b9eb425c9781d0a403503a63</t>
   </si>
   <si>
     <t>Water_EaTai</t>
@@ -235,7 +235,7 @@
     <t>Water_Fen_Fenix</t>
   </si>
   <si>
-    <t>1b111459c1604194b8340b08badad543</t>
+    <t>273eae91cfbc449abc2e5ab2f82e772c</t>
   </si>
   <si>
     <t>Water_Fen</t>
@@ -247,7 +247,7 @@
     <t>Water_Hom_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>d8e6a160643b4669bad7f1acfeacc7a7</t>
+    <t>ce02a2293fdc4dd29f6a3aa5f9e2937b</t>
   </si>
   <si>
     <t>Water_Hom</t>
@@ -268,7 +268,7 @@
     <t>Water_Kach_Kachi</t>
   </si>
   <si>
-    <t>49537d4d105b48f5b546bf6fc2c9ce45</t>
+    <t>252c53f1b8094ec0a903445e92dd3ab6</t>
   </si>
   <si>
     <t>Water_Kach</t>
@@ -280,7 +280,7 @@
     <t>Water_Lak_Lakkor Tso</t>
   </si>
   <si>
-    <t>0abb309ce46e4b4bac17a363bd91d2ed</t>
+    <t>3d5b154b6ea245d0a25d0e96ea8726a0</t>
   </si>
   <si>
     <t>Water_Lak</t>
@@ -292,7 +292,7 @@
     <t>Water_Mari_Maricunga</t>
   </si>
   <si>
-    <t>343b8eecf93240ae8f53acabd9e66220</t>
+    <t>9bfdd783653d41eeae6922caed5f322b</t>
   </si>
   <si>
     <t>Water_Mari</t>
@@ -304,7 +304,7 @@
     <t>Water_Ola_Salar de Olaroz</t>
   </si>
   <si>
-    <t>170fdd89d1ef4bf8a9aaaab0363727a3</t>
+    <t>5ba76416774c4a7b87a8988d1475d068</t>
   </si>
   <si>
     <t>Water_Ola</t>
@@ -316,7 +316,7 @@
     <t>Water_Pas_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>554935822e524f5aa1b0549a7c5398da</t>
+    <t>221f053e12494a899b2454f5904b83d6</t>
   </si>
   <si>
     <t>Water_Pas</t>
@@ -331,7 +331,7 @@
     <t>Water_Poz_Pozuelos</t>
   </si>
   <si>
-    <t>77e401faedf3448f8460745397911f9f</t>
+    <t>5258835e45e544b58281986158ef84f0</t>
   </si>
   <si>
     <t>Water_Poz</t>
@@ -346,7 +346,7 @@
     <t>Water_Rin_Salar del Rincon</t>
   </si>
   <si>
-    <t>ff1323ae49234997a1a23d9535cf3224</t>
+    <t>1203d095372740938783f54d8f25f003</t>
   </si>
   <si>
     <t>Water_Rin</t>
@@ -358,7 +358,7 @@
     <t>Water_Sil_Silver Peak</t>
   </si>
   <si>
-    <t>e1b2b3f79fab43248112fbce70a7b4c1</t>
+    <t>92f422be95a6475d8981464744255400</t>
   </si>
   <si>
     <t>US-WECC</t>
@@ -373,7 +373,7 @@
     <t>Water_Tol_Salar de Tolillar</t>
   </si>
   <si>
-    <t>1da4ff9773ad4883963efe9df3cf7a9a</t>
+    <t>9aa21cb818214d66be4878f2ee523f61</t>
   </si>
   <si>
     <t>Water_Tol</t>
@@ -385,7 +385,7 @@
     <t>Water_TresQ_Tres Quebradas</t>
   </si>
   <si>
-    <t>4f03812dec544597829517dab845f2e3</t>
+    <t>f924a81e4de34b549ce853b4cb06da3c</t>
   </si>
   <si>
     <t>Water_TresQ</t>
@@ -397,7 +397,7 @@
     <t>Water_URG_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>899cb25fa6474b77b782a87028947445</t>
+    <t>bc939f122857485ab866bb67a9b4b444</t>
   </si>
   <si>
     <t>Water_URG</t>
@@ -412,7 +412,7 @@
     <t>Water_Uyu_Salar de Uyuni</t>
   </si>
   <si>
-    <t>03948bb6f72648f28aa2047b3c547fbc</t>
+    <t>39f2ce29e1504b2292a3056c1dfc432e</t>
   </si>
   <si>
     <t>BO</t>
@@ -427,7 +427,7 @@
     <t>Water_Vid_Sal de Vida</t>
   </si>
   <si>
-    <t>c432ab78d8af439281078a94e149f3b9</t>
+    <t>9019eeec5daf48be9d53eabe1395a383</t>
   </si>
   <si>
     <t>Water_Vid</t>
@@ -439,7 +439,7 @@
     <t>Water_Yilip_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>63ae3a098ad740ce8ac03a92c6a1a2a5</t>
+    <t>d0cc4d98ae4c4ff4a4f1ebf50d672534</t>
   </si>
   <si>
     <t>Water_Yilip</t>
@@ -451,7 +451,7 @@
     <t>Water_Zha_Zhabuye</t>
   </si>
   <si>
-    <t>26edc309913a4dfeb1eeeb7b91c96879</t>
+    <t>f1027c3670814160ade2d68737521eca</t>
   </si>
   <si>
     <t>Water_Zha</t>
@@ -463,7 +463,7 @@
     <t>df_B_removal_orgsolvent_Maricunga</t>
   </si>
   <si>
-    <t>c1960eba128a448fa9595c6760b26499</t>
+    <t>07460306534b47b5a02e476099ae8870</t>
   </si>
   <si>
     <t>df_B_removal_orgsolvent</t>
@@ -511,7 +511,7 @@
     <t>df_B_removal_orgsolvent_Salar de Atacama</t>
   </si>
   <si>
-    <t>786ebf69e9a64100876c4637fcd64327</t>
+    <t>bb11a8f50c6b457d889e1b1b4039bd26</t>
   </si>
   <si>
     <t>df_transport_brine_Salar de Atacama</t>
@@ -523,7 +523,7 @@
     <t>df_B_removal_orgsolvent_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>4bc906c6d32645d6a5d91b845424ef26</t>
+    <t>341df9f5527d47b7b53c654ea64b5d48</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar de Cauchari-Olaroz</t>
@@ -532,19 +532,19 @@
     <t>df_B_removal_orgsolvent_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>b961fd6b283a41ab907d727537505670</t>
+    <t>ca9a930aa76f457eb14c009209e8c48c</t>
   </si>
   <si>
     <t>df_B_removal_orgsolvent_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>a4941dce3847443c9bb3fcfd3f561615</t>
+    <t>e34f659c60454facab79c0e9d1504b7b</t>
   </si>
   <si>
     <t>df_B_removal_orgsolvent_Tres Quebradas</t>
   </si>
   <si>
-    <t>c3f8e467b2e24575a8e969b1b97e349c</t>
+    <t>5555aa8d646648ebad41a6d36502a3e6</t>
   </si>
   <si>
     <t>df_transport_brine_Tres Quebradas</t>
@@ -553,7 +553,7 @@
     <t>df_CaMg_removal_sodiumhydrox_Sal de Vida</t>
   </si>
   <si>
-    <t>494f567d9a3749b4854a41bd2ee3f3a3</t>
+    <t>5672580887ab43e9b77d451c05666b53</t>
   </si>
   <si>
     <t>df_CaMg_removal_sodiumhydrox</t>
@@ -562,7 +562,7 @@
     <t>df_CaMg_removal_sodiumhydrox_Tres Quebradas</t>
   </si>
   <si>
-    <t>0d4ce199e6e8487e864eaf89ab9bdbf1</t>
+    <t>04c6789a18cd49e8b25b4888a9fb5436</t>
   </si>
   <si>
     <t>df_centrifuge_purification_sodaash_Tres Quebradas</t>
@@ -586,7 +586,7 @@
     <t>df_CaMg_removal_sodiumhydrox_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>3da9328e808e46f2a62d88241f030e56</t>
+    <t>0309f2244cc64909b2cf408b76c2f70a</t>
   </si>
   <si>
     <t>df_Li_adsorption_Upper Rhine Graben</t>
@@ -604,7 +604,7 @@
     <t>df_DLE_evaporation_ponds_Chaerhan</t>
   </si>
   <si>
-    <t>df7523e2462242b7bd4430fe4e2d6f61</t>
+    <t>299be317557f427d8e4e876d3902c5aa</t>
   </si>
   <si>
     <t>df_DLE_evaporation_ponds</t>
@@ -643,7 +643,7 @@
     <t>df_DLE_evaporation_ponds_Fenix</t>
   </si>
   <si>
-    <t>5deab68816e742929cdcd2c0ff49c976</t>
+    <t>d676acd8b32a47dba21a9790fa9009d1</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Fenix</t>
@@ -661,7 +661,7 @@
     <t>df_DLE_evaporation_ponds_Kachi</t>
   </si>
   <si>
-    <t>f42918f07bb942d589e06202fb93359c</t>
+    <t>87d9458b4c0042cca2ce71efb00173f9</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Kachi</t>
@@ -676,7 +676,7 @@
     <t>df_DLE_evaporation_ponds_Lakkor Tso</t>
   </si>
   <si>
-    <t>a96c82750cee447eb6ded98a9d473646</t>
+    <t>2c80fb4bb7cf4bea83d2276cf4dd6908</t>
   </si>
   <si>
     <t>df_reverse_osmosis_Lakkor Tso</t>
@@ -691,13 +691,13 @@
     <t>df_DLE_evaporation_ponds_Pozuelos</t>
   </si>
   <si>
-    <t>9951a0884f16465e87f9479734c24804</t>
+    <t>9658245fa6904f3ba25607b7a37f79a8</t>
   </si>
   <si>
     <t>df_DLE_evaporation_ponds_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>5b4e42f6471d4241a92c59f929cbab9a</t>
+    <t>8d47c44547414007b02ecf9a2c3cd7bf</t>
   </si>
   <si>
     <t>df_reverse_osmosis_Qinghai Yiliping</t>
@@ -712,7 +712,7 @@
     <t>df_DLE_evaporation_ponds_Sal de los Angeles</t>
   </si>
   <si>
-    <t>8fff05e837844ca793ddca15277cd614</t>
+    <t>e38b1fb5b33642548d0bb2820f6fc5a3</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Sal de los Angeles</t>
@@ -727,13 +727,13 @@
     <t>df_DLE_evaporation_ponds_Salar de Arizaro</t>
   </si>
   <si>
-    <t>a2cdba1f82dc467ba4e228d44de2181a</t>
+    <t>29e65c153e95401fba8b1b57a081461d</t>
   </si>
   <si>
     <t>df_DLE_evaporation_ponds_Salar de Centenario</t>
   </si>
   <si>
-    <t>a378cbd9f8dc4ff7b267963932f79681</t>
+    <t>a8fc41c3f3f246fd88878711e5a912a0</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Salar de Centenario</t>
@@ -748,13 +748,13 @@
     <t>df_DLE_evaporation_ponds_Salar de Tolillar</t>
   </si>
   <si>
-    <t>f2e9d320b2fb4cac8d252eb7ec8d09ac</t>
+    <t>a0373e754ce04936b55b060bc6927505</t>
   </si>
   <si>
     <t>df_DLE_evaporation_ponds_Salar de Uyuni</t>
   </si>
   <si>
-    <t>ef83442228374b1a88c606d075bd8770</t>
+    <t>48ace7d202034801a30d973573287222</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Salar de Uyuni</t>
@@ -769,7 +769,7 @@
     <t>df_DLE_evaporation_ponds_Salar del Rincon</t>
   </si>
   <si>
-    <t>9726aa9c269e4bbeb1bf9137cb3077e8</t>
+    <t>e664a098ffa046bbac59e091e09657ae</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Salar del Rincon</t>
@@ -784,7 +784,7 @@
     <t>df_Li_adsorption_Chaerhan</t>
   </si>
   <si>
-    <t>5ae4a4710f864efdaf9c27bd4193ca1c</t>
+    <t>2234db1f5b9b4ee69561a7262693efac</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Chaerhan</t>
@@ -799,7 +799,7 @@
     <t>df_Li_adsorption_East Taijinar</t>
   </si>
   <si>
-    <t>c144a8dc47e148e6981384fb4d8b5d78</t>
+    <t>d197949dc6e644f8be62c49023049825</t>
   </si>
   <si>
     <t>df_acidification_East Taijinar</t>
@@ -811,7 +811,7 @@
     <t>df_Li_adsorption_Fenix</t>
   </si>
   <si>
-    <t>6bb44689613b42d0b37cd5caea04784a</t>
+    <t>abeda27e2a534f308e019b3ca8dc8148</t>
   </si>
   <si>
     <t>df_acidification_Fenix</t>
@@ -820,7 +820,7 @@
     <t>df_Li_adsorption_Kachi</t>
   </si>
   <si>
-    <t>a313a42878d74bbaa3b707efd5756a06</t>
+    <t>6bd6fda6440349e1ab18579c98b58975</t>
   </si>
   <si>
     <t>df_acidification_Kachi</t>
@@ -829,7 +829,7 @@
     <t>df_Li_adsorption_Lakkor Tso</t>
   </si>
   <si>
-    <t>22d5692b49bc477694488cc514a33dcf</t>
+    <t>b46b86a391a34a61b1df118eba0fa40f</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Lakkor Tso</t>
@@ -838,13 +838,13 @@
     <t>df_Li_adsorption_Pozuelos</t>
   </si>
   <si>
-    <t>0ef2554e2a374c5a9938631af049f3cf</t>
+    <t>952dee573f994d2f979598e60d64753e</t>
   </si>
   <si>
     <t>df_Li_adsorption_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>74a825eadb044a1ba17948163ece0276</t>
+    <t>d6191c58da6d4ac9a55b7fe2137c14ca</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Qinghai Yiliping</t>
@@ -853,7 +853,7 @@
     <t>df_Li_adsorption_Sal de los Angeles</t>
   </si>
   <si>
-    <t>003f98db3d854065883e9c21783c5bb4</t>
+    <t>ec12bf0857814ce7881a35baca9bb9f1</t>
   </si>
   <si>
     <t>df_acidification_Sal de los Angeles</t>
@@ -862,13 +862,13 @@
     <t>df_Li_adsorption_Salar de Arizaro</t>
   </si>
   <si>
-    <t>1f53615c143542afb22b6117a1d1b946</t>
+    <t>e50fcaf8a2aa4a2787e448b8a10caad2</t>
   </si>
   <si>
     <t>df_Li_adsorption_Salar de Centenario</t>
   </si>
   <si>
-    <t>13388b3a630f49f8a93d34563a1ebd8b</t>
+    <t>202768eb2eec4d7ab15a4063bd7a83c9</t>
   </si>
   <si>
     <t>df_acidification_Salar de Centenario</t>
@@ -877,13 +877,13 @@
     <t>df_Li_adsorption_Salar de Tolillar</t>
   </si>
   <si>
-    <t>60d664ecda0348d7b1d0da7a89c0c597</t>
+    <t>56e75d38f9ad4fe882c4322fc1dbbcd1</t>
   </si>
   <si>
     <t>df_Li_adsorption_Salar de Uyuni</t>
   </si>
   <si>
-    <t>b19858474b084871be7af3128339188f</t>
+    <t>f9a370e3a3814e86a58c56b7f4ebeb8c</t>
   </si>
   <si>
     <t>df_acidification_Salar de Uyuni</t>
@@ -892,7 +892,7 @@
     <t>df_Li_adsorption_Salar del Rincon</t>
   </si>
   <si>
-    <t>3761443a7fce461882cac5d12e9d548f</t>
+    <t>dc30f607626b4a8486f4713faaa81c07</t>
   </si>
   <si>
     <t>df_acidification_Salar del Rincon</t>
@@ -904,7 +904,7 @@
     <t>heat, central or small-scale, other than natural gas</t>
   </si>
   <si>
-    <t>a7b54018dcf54c98b50450b14a52f719</t>
+    <t>911cc080446a46df8331bd04dccf895c</t>
   </si>
   <si>
     <t>df_acidification_Upper Rhine Graben</t>
@@ -913,7 +913,7 @@
     <t>df_Liprec_BG_Chaerhan</t>
   </si>
   <si>
-    <t>a49c3254f48c4352a5fe36c0ca1de953</t>
+    <t>1077b521ba0245e0a7191936203cbc8f</t>
   </si>
   <si>
     <t>df_Liprec_BG</t>
@@ -928,7 +928,7 @@
     <t>df_Liprec_BG_East Taijinar</t>
   </si>
   <si>
-    <t>f70ca80990e144f8bf14c56e5c24c26d</t>
+    <t>55da9d6474b947a59bc6d9523a50bfa4</t>
   </si>
   <si>
     <t>df_dissolution_East Taijinar</t>
@@ -937,7 +937,7 @@
     <t>df_Liprec_BG_Fenix</t>
   </si>
   <si>
-    <t>f104b7666bb7488ba3c6b888f245748f</t>
+    <t>b1191c887b804a2ab3394b2f1ccf5bd2</t>
   </si>
   <si>
     <t>df_dissolution_Fenix</t>
@@ -946,7 +946,7 @@
     <t>df_Liprec_BG_Kachi</t>
   </si>
   <si>
-    <t>b25aa714f9084f3587272c00a106841e</t>
+    <t>4e3bc83ae26c46f5b352497b5d643ce6</t>
   </si>
   <si>
     <t>df_dissolution_Kachi</t>
@@ -955,7 +955,7 @@
     <t>df_Liprec_BG_Lakkor Tso</t>
   </si>
   <si>
-    <t>72bd1395c3634e7f804cbce301c0bbdd</t>
+    <t>aa5dff62cb43498098e196329bc6dea3</t>
   </si>
   <si>
     <t>df_dissolution_Lakkor Tso</t>
@@ -964,7 +964,7 @@
     <t>df_Liprec_BG_Maricunga</t>
   </si>
   <si>
-    <t>8182db6003af406aa09239bd9ea8db3f</t>
+    <t>080b87ba3dee4c0cb2783f5bf249bfd0</t>
   </si>
   <si>
     <t>df_dissolution_Maricunga</t>
@@ -979,13 +979,13 @@
     <t>df_Liprec_BG_Pozuelos</t>
   </si>
   <si>
-    <t>71d0ea0f198642bd9efea5735a7fe058</t>
+    <t>0c836ea946e84d0c86825280b5ef2bf0</t>
   </si>
   <si>
     <t>df_Liprec_BG_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>d0ee981adf6b435ba65f4f1f9152efe3</t>
+    <t>b4f8974389bc416c899b7f8a59451887</t>
   </si>
   <si>
     <t>df_dissolution_Qinghai Yiliping</t>
@@ -994,13 +994,13 @@
     <t>df_Liprec_BG_Sal de Vida</t>
   </si>
   <si>
-    <t>7052b3a8c5a44e84acbacd1118a77f6c</t>
+    <t>ee1876c3ce8a40bfa0b7347d6b5f0e05</t>
   </si>
   <si>
     <t>df_Liprec_BG_Sal de los Angeles</t>
   </si>
   <si>
-    <t>993c1fa2e9614fd3af7583fa5d2a0766</t>
+    <t>7405f0ec48394396a6a24daf4f26bd9b</t>
   </si>
   <si>
     <t>df_dissolution_Sal de los Angeles</t>
@@ -1009,13 +1009,13 @@
     <t>df_Liprec_BG_Salar de Arizaro</t>
   </si>
   <si>
-    <t>91a984309b4745e69881663fd538cdf5</t>
+    <t>923f78a6a387422abbf69e45e6bc03b2</t>
   </si>
   <si>
     <t>df_Liprec_BG_Salar de Atacama</t>
   </si>
   <si>
-    <t>025eceeb1d0d43c7a843c878e38b6b12</t>
+    <t>d1d2995216b04349a621625a362fd95d</t>
   </si>
   <si>
     <t>df_dissolution_Salar de Atacama</t>
@@ -1024,7 +1024,7 @@
     <t>df_Liprec_BG_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>41e538731a19490390fb25d487781a1e</t>
+    <t>5551239ab46f43cbbce26ccbb8dbd880</t>
   </si>
   <si>
     <t>df_dissolution_Salar de Cauchari-Olaroz</t>
@@ -1033,7 +1033,7 @@
     <t>df_Liprec_BG_Salar de Centenario</t>
   </si>
   <si>
-    <t>93b9b6e93f574d70a4f32a0a01921ae3</t>
+    <t>6e7b5302bea54de7b24babe77fdaec98</t>
   </si>
   <si>
     <t>df_dissolution_Salar de Centenario</t>
@@ -1042,7 +1042,7 @@
     <t>df_Liprec_BG_Salar de Olaroz</t>
   </si>
   <si>
-    <t>a780c1c65a834debaa2fa016e20146ab</t>
+    <t>31266e034827481791f69b785e6870d0</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Salar de Olaroz</t>
@@ -1051,19 +1051,19 @@
     <t>df_Liprec_BG_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>fb3e814df514455fae8cfbe981f79d3e</t>
+    <t>7837f05726bf4aa8abb5b17ce51a204b</t>
   </si>
   <si>
     <t>df_Liprec_BG_Salar de Tolillar</t>
   </si>
   <si>
-    <t>35fc4251654148a9a8db2eacc6cf05d5</t>
+    <t>6793bac6e86442f987a716c38d166e70</t>
   </si>
   <si>
     <t>df_Liprec_BG_Salar de Uyuni</t>
   </si>
   <si>
-    <t>9fee7eb2802045b2aeecd9a82daede0a</t>
+    <t>3044ea3cea084d9d8518b81d2be9b4e4</t>
   </si>
   <si>
     <t>df_dissolution_Salar de Uyuni</t>
@@ -1072,13 +1072,13 @@
     <t>df_Liprec_BG_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>733db39a98df48239f33a82fcd069185</t>
+    <t>a942528819d640c7a1a4260d03cb1065</t>
   </si>
   <si>
     <t>df_Liprec_BG_Salar del Rincon</t>
   </si>
   <si>
-    <t>db6679fb25c3448c8d5f63384e28147f</t>
+    <t>0692b71c42884b4cad129b32aea4a412</t>
   </si>
   <si>
     <t>df_dissolution_Salar del Rincon</t>
@@ -1087,7 +1087,7 @@
     <t>df_Liprec_BG_Silver Peak</t>
   </si>
   <si>
-    <t>68cc57d99d7e45c2890a98e67657a38d</t>
+    <t>b42e4c71375949c79507250d7d2b03dc</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Silver Peak</t>
@@ -1099,7 +1099,7 @@
     <t>df_Liprec_BG_Tres Quebradas</t>
   </si>
   <si>
-    <t>47df6fc0e0774ebab37a89cc93f6db96</t>
+    <t>a38ff368055c43159aeef726613fae5b</t>
   </si>
   <si>
     <t>df_dissolution_Tres Quebradas</t>
@@ -1108,7 +1108,7 @@
     <t>df_Liprec_BG_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>1cdab5c88f1c489c860346e16e0099c3</t>
+    <t>acc14cc6d2734c1cb42d8010dda9065f</t>
   </si>
   <si>
     <t>df_dissolution_Upper Rhine Graben</t>
@@ -1117,7 +1117,7 @@
     <t>df_Liprec_BG_Zhabuye</t>
   </si>
   <si>
-    <t>30f1f63450a34ff6b7aa2a47d78a3b74</t>
+    <t>034e845d2e404fcd8425f3ea46a39b07</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Zhabuye</t>
@@ -1126,7 +1126,7 @@
     <t>df_Liprec_TG_Chaerhan</t>
   </si>
   <si>
-    <t>a8cd41ab465d4f94a5edae51d73f9772</t>
+    <t>a5f4ba5b68994ae0beb03b20b8004f80</t>
   </si>
   <si>
     <t>df_Liprec_TG</t>
@@ -1135,7 +1135,7 @@
     <t>df_Liprec_TG_East Taijinar</t>
   </si>
   <si>
-    <t>bd6b4ecbb82948bbadaaa40c4a17f554</t>
+    <t>b58a0171ac3d4058b0a99c1298dfaaed</t>
   </si>
   <si>
     <t>df_reverse_osmosis_East Taijinar</t>
@@ -1144,25 +1144,25 @@
     <t>df_Liprec_TG_Fenix</t>
   </si>
   <si>
-    <t>47399de470e84e7285550542893f7845</t>
+    <t>92cee059d9a64a69b9aa2c7a57da3251</t>
   </si>
   <si>
     <t>df_Liprec_TG_Kachi</t>
   </si>
   <si>
-    <t>031dc09a44b943c2b986e4a3e4745b42</t>
+    <t>cfa6471e79344de48c6912cef86d8bb5</t>
   </si>
   <si>
     <t>df_Liprec_TG_Lakkor Tso</t>
   </si>
   <si>
-    <t>82d93e317de9400fb769e9b0f985e5f8</t>
+    <t>c2f249dc6d5f41bfa2ccae699661a0b2</t>
   </si>
   <si>
     <t>df_Liprec_TG_Maricunga</t>
   </si>
   <si>
-    <t>32ff674b08a745c0bf35be1cb8324485</t>
+    <t>b4d530eed8a14efc83c6ceaf6ee1ad10</t>
   </si>
   <si>
     <t>df_ion_exchange_H_Maricunga</t>
@@ -1174,37 +1174,37 @@
     <t>df_Liprec_TG_Pozuelos</t>
   </si>
   <si>
-    <t>c748cdcd65474675842659178c09d78d</t>
+    <t>d13f645f839a487790823829d148ab47</t>
   </si>
   <si>
     <t>df_Liprec_TG_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>1ee6b5ec7ff04db0bde22a5e9be751a7</t>
+    <t>7fe6874deb40405b81efc5ef90e62ab4</t>
   </si>
   <si>
     <t>df_Liprec_TG_Sal de Vida</t>
   </si>
   <si>
-    <t>572c8cb9c8cc46e09538d1c32fce5ac9</t>
+    <t>540494b95d044b1b86a392dbb423157e</t>
   </si>
   <si>
     <t>df_Liprec_TG_Sal de los Angeles</t>
   </si>
   <si>
-    <t>e27e0cdb86ad4e658d21d54143144021</t>
+    <t>11068b7e325641fdaf9a72ac66ea0444</t>
   </si>
   <si>
     <t>df_Liprec_TG_Salar de Arizaro</t>
   </si>
   <si>
-    <t>c0aebb5604814870b28aa84bc739aa47</t>
+    <t>abab839c835b4dfebda2a0e29595ec98</t>
   </si>
   <si>
     <t>df_Liprec_TG_Salar de Atacama</t>
   </si>
   <si>
-    <t>68d72a1dd2fa4d3c81f9a7066c806cfb</t>
+    <t>49eb4cecc4a54038bb858a12b3a456fc</t>
   </si>
   <si>
     <t>df_centrifuge_purification_quicklime_Salar de Atacama</t>
@@ -1216,7 +1216,7 @@
     <t>df_Liprec_TG_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>d9bdaa9982764161ac319a28809935cc</t>
+    <t>d2f7a7083b8f431ba7db46d2b46b3272</t>
   </si>
   <si>
     <t>df_triple_evaporator_Salar de Cauchari-Olaroz</t>
@@ -1228,13 +1228,13 @@
     <t>df_Liprec_TG_Salar de Centenario</t>
   </si>
   <si>
-    <t>b992942bf5454797b0bb68e7d84d92ba</t>
+    <t>6f9e39158dae4faa8d8a7139b9803403</t>
   </si>
   <si>
     <t>df_Liprec_TG_Salar de Olaroz</t>
   </si>
   <si>
-    <t>56d87af257754c7e982d90a2eaf44e4e</t>
+    <t>b0887a7fead546cfba0e2d595656857e</t>
   </si>
   <si>
     <t>df_centrifuge_general_1_Salar de Olaroz</t>
@@ -1246,37 +1246,37 @@
     <t>df_Liprec_TG_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>e0a35f86c3d746969be768aff677589e</t>
+    <t>2e822396737d4e6cb67c2cc87a34417a</t>
   </si>
   <si>
     <t>df_Liprec_TG_Salar de Tolillar</t>
   </si>
   <si>
-    <t>e9912bd9fb4f4a31a2a1487d230466fc</t>
+    <t>b8c1ef717f094cb78547b94b85e75b51</t>
   </si>
   <si>
     <t>df_Liprec_TG_Salar de Uyuni</t>
   </si>
   <si>
-    <t>430e056b04da412c830c3d983c3b8c29</t>
+    <t>ce970f594b414e84bc0f9748afa5fd11</t>
   </si>
   <si>
     <t>df_Liprec_TG_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>7fd7d6676a354154937d74a0f32591e7</t>
+    <t>c9a6da91c454415aab9d1f040793caf6</t>
   </si>
   <si>
     <t>df_Liprec_TG_Salar del Rincon</t>
   </si>
   <si>
-    <t>85020e4c018049a696e3654ec2dfe1e3</t>
+    <t>e829d15c61834a21ae337b8e8e5d62c5</t>
   </si>
   <si>
     <t>df_Liprec_TG_Silver Peak</t>
   </si>
   <si>
-    <t>8d30335660d2492ba793ffbb99fb4648</t>
+    <t>529d1e6a5637467aa125610ca5b54581</t>
   </si>
   <si>
     <t>df_centrifuge_general_1_Silver Peak</t>
@@ -1285,7 +1285,7 @@
     <t>df_Liprec_TG_Tres Quebradas</t>
   </si>
   <si>
-    <t>399ee3bb943047cfaebff82faed1baf7</t>
+    <t>3f67022590864ac2a5daf08bc4d19e28</t>
   </si>
   <si>
     <t>df_centrifuge_general_1_Tres Quebradas</t>
@@ -1294,7 +1294,7 @@
     <t>df_Liprec_TG_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>3712c7037f18468a9f52fa431c9fc3a9</t>
+    <t>74f047725ac54087a0755c7151c8be71</t>
   </si>
   <si>
     <t>df_triple_evaporator_Upper Rhine Graben</t>
@@ -1303,7 +1303,7 @@
     <t>df_Mg_removal_quicklime_East Taijinar</t>
   </si>
   <si>
-    <t>2ae4598a7e1249baa9ceb54961bd5ae2</t>
+    <t>6a6da14c575d4fb8b9d027a2cdb2f1cc</t>
   </si>
   <si>
     <t>df_Mg_removal_quicklime</t>
@@ -1321,7 +1321,7 @@
     <t>df_Mg_removal_quicklime_Maricunga</t>
   </si>
   <si>
-    <t>ad402c22b50a491880d157474ff76090</t>
+    <t>189a36a5c64b4fc79e890f59a1f521d7</t>
   </si>
   <si>
     <t>df_centrifuge_purification_sodaash_Maricunga</t>
@@ -1330,7 +1330,7 @@
     <t>df_Mg_removal_quicklime_Salar de Atacama</t>
   </si>
   <si>
-    <t>2f572d8c03e349a99ad6d3c7cb104a77</t>
+    <t>3d7aacda2f0f4cad8c7989555f7a1cf8</t>
   </si>
   <si>
     <t>df_centrifuge_purification_sodaash_Salar de Atacama</t>
@@ -1339,7 +1339,7 @@
     <t>df_Mg_removal_quicklime_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>3b80f9a9fd704cfcbdcf2fd9e0812dbc</t>
+    <t>e20d2af9a0d043c5bf19942b89edc440</t>
   </si>
   <si>
     <t>df_centrifuge_purification_sodaash_Salar de Cauchari-Olaroz</t>
@@ -1348,19 +1348,19 @@
     <t>df_Mg_removal_quicklime_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>3b3e46171f09452e98c2a285ec504434</t>
+    <t>a19d6abf016a4be9a239ffefd6caa40f</t>
   </si>
   <si>
     <t>df_Mg_removal_quicklime_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>c4f72973c0f747aa8e83221ed2490c0a</t>
+    <t>fb0f5ab0f0884f6d89dd6051eb10450b</t>
   </si>
   <si>
     <t>df_Mg_removal_sodaash_Fenix</t>
   </si>
   <si>
-    <t>e4d557ebec294cbaa14daec9777b674f</t>
+    <t>f35ccd8bd46145feaf174f7ed426c9ce</t>
   </si>
   <si>
     <t>df_Mg_removal_sodaash</t>
@@ -1372,7 +1372,7 @@
     <t>df_Mg_removal_sodaash_Kachi</t>
   </si>
   <si>
-    <t>2007de3978e24014b6b3b01a21141670</t>
+    <t>8941e829bbd04e7cac283c7ef3c6d265</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Kachi</t>
@@ -1381,7 +1381,7 @@
     <t>df_Mg_removal_sodaash_Maricunga</t>
   </si>
   <si>
-    <t>0f2c9d3f4d604b299da12f6c867c1daf</t>
+    <t>cf89e445a3cf4b20a385b3fb2f4ce92e</t>
   </si>
   <si>
     <t>df_centrifuge_general_1_Maricunga</t>
@@ -1390,19 +1390,19 @@
     <t>df_Mg_removal_sodaash_Pozuelos</t>
   </si>
   <si>
-    <t>b40a4b030db741748a9985e85b374011</t>
+    <t>8352c6f0fa834e9b934d38b991390283</t>
   </si>
   <si>
     <t>df_Mg_removal_sodaash_Sal de Vida</t>
   </si>
   <si>
-    <t>b51a501448f04318a964aa26db387766</t>
+    <t>ff6e7e654ad74659ab0a61babc36bb7a</t>
   </si>
   <si>
     <t>df_Mg_removal_sodaash_Sal de los Angeles</t>
   </si>
   <si>
-    <t>ffb16296242b46239f6a93735b6420f3</t>
+    <t>e15ba3160d3641c398e6a4dbca94adc6</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Sal de los Angeles</t>
@@ -1411,13 +1411,13 @@
     <t>df_Mg_removal_sodaash_Salar de Arizaro</t>
   </si>
   <si>
-    <t>e896387450714546971c569554ce9b4f</t>
+    <t>22fb299d6135494796abd5a10b58f166</t>
   </si>
   <si>
     <t>df_Mg_removal_sodaash_Salar de Atacama</t>
   </si>
   <si>
-    <t>f295c69e9c194db0aaea56c3e383448d</t>
+    <t>c0d8433e42d34730bbc8e45b49291ccc</t>
   </si>
   <si>
     <t>df_centrifuge_general_1_Salar de Atacama</t>
@@ -1426,13 +1426,13 @@
     <t>df_Mg_removal_sodaash_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>304337c4023648d1900f89b386459061</t>
+    <t>2cbe6cd094d245d887a0cd3779bde5ed</t>
   </si>
   <si>
     <t>df_Mg_removal_sodaash_Salar de Centenario</t>
   </si>
   <si>
-    <t>28217f044ee94642a8991d1bea5c85da</t>
+    <t>f92fd7f8a8864d18bc269d3dc7e89ed7</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar de Centenario</t>
@@ -1441,19 +1441,19 @@
     <t>df_Mg_removal_sodaash_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>c659c2be3abc4e238c7aff7870787a87</t>
+    <t>402fa1f0c809475d95ba086f0480f223</t>
   </si>
   <si>
     <t>df_Mg_removal_sodaash_Salar de Tolillar</t>
   </si>
   <si>
-    <t>79eebf14db8644b9b3c217db0ffb1481</t>
+    <t>9363ce155ffd45c09ba4a735cc574952</t>
   </si>
   <si>
     <t>df_Mg_removal_sodaash_Salar de Uyuni</t>
   </si>
   <si>
-    <t>17e4dd4ebc01444895fce1bc95438d6a</t>
+    <t>d72d754c50cc489faafd9df72008e1e3</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar de Uyuni</t>
@@ -1462,13 +1462,13 @@
     <t>df_Mg_removal_sodaash_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>4098e03fe4d1495e89b21beb31719777</t>
+    <t>92f3f327e0c84bad931c68ea4273c46b</t>
   </si>
   <si>
     <t>df_Mg_removal_sodaash_Salar del Rincon</t>
   </si>
   <si>
-    <t>c1c97ee9dd024f7785d7d709e636d3eb</t>
+    <t>7e42dfc085fb4ef8b2cda0dd8a52fad1</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar del Rincon</t>
@@ -1477,13 +1477,13 @@
     <t>df_Mg_removal_sodaash_Tres Quebradas</t>
   </si>
   <si>
-    <t>ea39afa7257e4268aa23cdaba1748c83</t>
+    <t>09f894485a9c4f97981efa1991d9ee58</t>
   </si>
   <si>
     <t>df_MnZn_removal_lime_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>d2c300dc25c24d409bc1deb7763ac3b9</t>
+    <t>43f1739bed7343d3a12c81e9d4478c8d</t>
   </si>
   <si>
     <t>df_MnZn_removal_lime</t>
@@ -1495,7 +1495,7 @@
     <t>df_SiFe_removal_limestone</t>
   </si>
   <si>
-    <t>46cb9dd4c86841a3a3ddb8da445aeb60</t>
+    <t>a32a9d1454b54cd581226038ad770092</t>
   </si>
   <si>
     <t>Lithium</t>
@@ -1507,7 +1507,7 @@
     <t>limestone, crushed, washed</t>
   </si>
   <si>
-    <t>f94362fac6e047fb82ddc9f70eb69093</t>
+    <t>ef1e8c7e648a46a4b76c86eb65fc8431</t>
   </si>
   <si>
     <t>df_sulfate_removal_calciumchloride_East Taijinar</t>
@@ -1516,49 +1516,49 @@
     <t>df_sulfate_removal_calciumchloride</t>
   </si>
   <si>
-    <t>85f8217f959749c38f50967e360dc0b2</t>
-  </si>
-  <si>
-    <t>e6225de6c9824d3baf69211337222e2f</t>
+    <t>f278a6f466ea43d4a45be380660604b5</t>
+  </si>
+  <si>
+    <t>3b6fcb68a88741e7bf63bdf9c3fe5cc0</t>
   </si>
   <si>
     <t>df_acidification_Pozuelos</t>
   </si>
   <si>
-    <t>b3f4d9a9f4a24ff6968051a835b0b0e3</t>
-  </si>
-  <si>
-    <t>f371acbb01f24ff0a4efe94bfad62915</t>
+    <t>2f595ae7aa6a405891cf943ea7042e4a</t>
+  </si>
+  <si>
+    <t>01e4cc88fe7149f78175ff733c5ef2ba</t>
   </si>
   <si>
     <t>df_acidification_Salar de Arizaro</t>
   </si>
   <si>
-    <t>56e2d8480fbb404cb66f5ed10360ce0d</t>
-  </si>
-  <si>
-    <t>19fdc902bd934ba99cca2a60a49eae2c</t>
+    <t>357d3bd26843491cb5522d15dd0d03da</t>
+  </si>
+  <si>
+    <t>f951c03c9e8443f4819ef6ebdbec0608</t>
   </si>
   <si>
     <t>df_acidification_Salar de Tolillar</t>
   </si>
   <si>
-    <t>fb399c36167944ecac8faaedb700f712</t>
-  </si>
-  <si>
-    <t>414d3e2b724140cba06522c35638d617</t>
-  </si>
-  <si>
-    <t>a0f6a5643dae4024a13466dd411780fc</t>
-  </si>
-  <si>
-    <t>e36216e4d9554ce2b906f8df08ed5890</t>
+    <t>497f44f0dcd04d26b3286f8d7fbee2e5</t>
+  </si>
+  <si>
+    <t>6fd1f34663d947cb9532fe53c8617d86</t>
+  </si>
+  <si>
+    <t>ab3c228175604d328d8c965db785568d</t>
+  </si>
+  <si>
+    <t>d8fba76a7c60479290cef19efabd5507</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Chaerhan</t>
   </si>
   <si>
-    <t>824079e515954904a40ea711adc9bfa5</t>
+    <t>30a16a1ef3024cfaa80d44ef4698cf16</t>
   </si>
   <si>
     <t>df_centrifuge_BG</t>
@@ -1567,7 +1567,7 @@
     <t>df_centrifuge_BG_East Taijinar</t>
   </si>
   <si>
-    <t>542fbeffd84c426b90ea9746e7899217</t>
+    <t>508388f5039745bf92f1bd245acb1adf</t>
   </si>
   <si>
     <t>waste_liquid_EaTai_East Taijinar</t>
@@ -1579,25 +1579,25 @@
     <t>df_centrifuge_BG_Fenix</t>
   </si>
   <si>
-    <t>85de1765c0134ab68404ac0fd1be2713</t>
+    <t>16cb0055e04048d284b3b2e543aba47a</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Kachi</t>
   </si>
   <si>
-    <t>10cf2edf0cc4426a8e3d6fc024e782aa</t>
+    <t>b6bfdc71e2384e1691934805a9cd9430</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Lakkor Tso</t>
   </si>
   <si>
-    <t>8cb64ab2f93e4c6c8a3ab92ed2b026e2</t>
+    <t>29ee9dc83a804539b12b357fd321c2ed</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Maricunga</t>
   </si>
   <si>
-    <t>2b25e0e4017449c1881e0b8cd2514929</t>
+    <t>49f7e69804094f5ca61ec1851ded1c80</t>
   </si>
   <si>
     <t>waste_liquid_Mari_Maricunga</t>
@@ -1609,37 +1609,37 @@
     <t>df_centrifuge_BG_Pozuelos</t>
   </si>
   <si>
-    <t>ccc7e5032d4443f2bb609e16a4808e08</t>
+    <t>5c80bf6520254c07a82eeeffe226efc5</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>3534d4b339fb4596b69a3668c5eb7466</t>
+    <t>64b0c1bedb6b4803bc1a808786d8671d</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Sal de Vida</t>
   </si>
   <si>
-    <t>6a017362e2d34504aa49372b785c0e4d</t>
+    <t>2dcc0f7b788b41e6b8ed36fc976aebdb</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Sal de los Angeles</t>
   </si>
   <si>
-    <t>8d4675df64264ba59c9c7786d2b473e2</t>
+    <t>1a19feccc30e441f9df114972a8acd38</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Salar de Arizaro</t>
   </si>
   <si>
-    <t>706e7b13732a49059fef759587434710</t>
+    <t>5e7b106b646d47e79c54402acca7fed4</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Salar de Atacama</t>
   </si>
   <si>
-    <t>f52e55da5f7f450ba57e5d7ba534dc2b</t>
+    <t>10340f5dfe0d4c50b0bdcf74c99d148f</t>
   </si>
   <si>
     <t>waste_liquid_Ata_Salar de Atacama</t>
@@ -1651,7 +1651,7 @@
     <t>df_centrifuge_BG_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>7b973c8b5d17400ab0edf8eff31b1730</t>
+    <t>a1c9ac79db6d407cb8de9d625762fc87</t>
   </si>
   <si>
     <t>waste_liquid_Cau_Salar de Cauchari-Olaroz</t>
@@ -1663,13 +1663,13 @@
     <t>df_centrifuge_BG_Salar de Centenario</t>
   </si>
   <si>
-    <t>56464eb975524a60b86c7c44ad4c4887</t>
+    <t>8081d186fa0340c4bf0f456444db2027</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Salar de Olaroz</t>
   </si>
   <si>
-    <t>9996a9d9d5594befa52e840d828b2319</t>
+    <t>f3cd68111a18409eb7604dfeb3df0635</t>
   </si>
   <si>
     <t>waste_liquid_Ola_Salar de Olaroz</t>
@@ -1681,37 +1681,37 @@
     <t>df_centrifuge_BG_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>d9e76eb513ee467cb2a39f995ba1e104</t>
+    <t>f5ef83cf4b864039a36474c7b7d75f53</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Salar de Tolillar</t>
   </si>
   <si>
-    <t>97e9ed435abd4013a44f2bb40220e9b2</t>
+    <t>4bfe0bd839c549ecaa493ff849996e9f</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Salar de Uyuni</t>
   </si>
   <si>
-    <t>df1ddd4acea7430a9a439f236ca19602</t>
+    <t>c65d7cf30ae541b0945a928916bc84a1</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>b76a9d86734443f49575259ca5d60a83</t>
+    <t>a72b163a658e4893b8b967ab6a7f97db</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Salar del Rincon</t>
   </si>
   <si>
-    <t>428cdb6e32e7418485594700993bdd1b</t>
+    <t>7d10d2c31c1a42a48bc0577066ed391e</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Silver Peak</t>
   </si>
   <si>
-    <t>952de989e74140b384c4b1338089b1ca</t>
+    <t>8c3294afd2c441a2aeda6df3c15283a6</t>
   </si>
   <si>
     <t>waste_liquid_Sil_Silver Peak</t>
@@ -1723,7 +1723,7 @@
     <t>df_centrifuge_BG_Tres Quebradas</t>
   </si>
   <si>
-    <t>df9ca44ed65241c8a9f8dcaccc6ec037</t>
+    <t>2f5cacb1a70c4765ac7f0fbffca4b0a6</t>
   </si>
   <si>
     <t>waste_liquid_TresQ_Tres Quebradas</t>
@@ -1735,13 +1735,13 @@
     <t>df_centrifuge_BG_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>ed6401ac350f466da5e40b9c815e436a</t>
+    <t>a7fba9eb9c92440ca6e88d349c4765a9</t>
   </si>
   <si>
     <t>df_centrifuge_BG_Zhabuye</t>
   </si>
   <si>
-    <t>9a4ec6425636439d88cc3daef1585bb8</t>
+    <t>3b49c7971b2e416caf4b5aa25e04cc7a</t>
   </si>
   <si>
     <t>waste_liquid_Zha_Zhabuye</t>
@@ -1753,7 +1753,7 @@
     <t>df_centrifuge_TG_Chaerhan</t>
   </si>
   <si>
-    <t>20289481d8214113a5cfac8d54d19582</t>
+    <t>be0eb5645fcd419a9f1fc9d797457f54</t>
   </si>
   <si>
     <t>df_centrifuge_TG</t>
@@ -1762,85 +1762,85 @@
     <t>df_centrifuge_TG_East Taijinar</t>
   </si>
   <si>
-    <t>0d0c3f9c48584cc28afdaa5973483814</t>
+    <t>701dfb7cf48441368e6060f1ded6e2de</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Fenix</t>
   </si>
   <si>
-    <t>2ff656d66a484a7bbb904b94655f5aa7</t>
+    <t>82a50864bba94971b035347b6922e6e2</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Kachi</t>
   </si>
   <si>
-    <t>9187c93f831b4e868a1e107aa9852d7c</t>
+    <t>99716cd2ec7643aaafab541a22083100</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Lakkor Tso</t>
   </si>
   <si>
-    <t>8b8c98791577442ea11acd94a4114369</t>
+    <t>a2ecd279a00e498f91fefa513dc27cfa</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Maricunga</t>
   </si>
   <si>
-    <t>e1b6aa1e1bbd45519c270ad5f11626d3</t>
+    <t>bf608df0236640e3b3470daff53b602b</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Pozuelos</t>
   </si>
   <si>
-    <t>06a87f510c7242e3a66858565713fb9e</t>
+    <t>3d6b92c0facd4f98bda8f92d09a7d1f2</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>034666ea4641431aa4886d24a421a813</t>
+    <t>70189a9e3a0b407e83798dce57886408</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Sal de Vida</t>
   </si>
   <si>
-    <t>1de33b403c7c4cc9846e271196a20051</t>
+    <t>7371f87da4f640a896b563aa3bea3944</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Sal de los Angeles</t>
   </si>
   <si>
-    <t>a21025c3249a46a99c3aa62bf5a4c126</t>
+    <t>71f5d30f96574a1d87182ad06de457b1</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Salar de Arizaro</t>
   </si>
   <si>
-    <t>1c2a7c990fe04597a3021f6521b76237</t>
+    <t>737b89a8442c423f9388b20d87fd318a</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Salar de Atacama</t>
   </si>
   <si>
-    <t>40f0d407be5a481d875a834a3c630ac6</t>
+    <t>585be158df8d4b3d84daeefae3a188b9</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>be6e63f259424679b53130296bc7d49c</t>
+    <t>bc96f0c22b5a4acb885dd2f542409b15</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Salar de Centenario</t>
   </si>
   <si>
-    <t>efe5ca0ded8f46eaa14bcd3ad2030dae</t>
+    <t>30a3e863aafb4574afb0f461a20f2047</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Salar de Olaroz</t>
   </si>
   <si>
-    <t>d276368d03644f728c509493e98d5009</t>
+    <t>35eccac44e244ace9150792b4eaa890a</t>
   </si>
   <si>
     <t>df_washing_TG_Salar de Olaroz</t>
@@ -1852,37 +1852,37 @@
     <t>df_centrifuge_TG_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>5e9e621b5e2143f1b307f360587ef7c6</t>
+    <t>137a9bb60df7498a8d9a4a15dd4d3713</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Salar de Tolillar</t>
   </si>
   <si>
-    <t>018569bb5a1b41f58134b9131827b5a1</t>
+    <t>6ce350ab744b4b7e83404d48aaf057d3</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Salar de Uyuni</t>
   </si>
   <si>
-    <t>c515fdc315b549809a6ae3461ad72668</t>
+    <t>b92c4427991f42ec949314d631cc2014</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>317b5443d9b04d728aa0f95992071a5c</t>
+    <t>f187dd3d9c8b4d568c075dbfd39a7923</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Salar del Rincon</t>
   </si>
   <si>
-    <t>4d7bc085ea864f2cae0495c7d7703ff7</t>
+    <t>90fb056db5754d57aa9326187ecd4ad6</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Silver Peak</t>
   </si>
   <si>
-    <t>afb455326bbc467da754498b712559e4</t>
+    <t>c896a24085cf401ca2a46c020446bbf9</t>
   </si>
   <si>
     <t>df_washing_TG_Silver Peak</t>
@@ -1891,22 +1891,22 @@
     <t>df_centrifuge_TG_Tres Quebradas</t>
   </si>
   <si>
-    <t>e8dccaffa4804736bc9120f6f06ad818</t>
+    <t>6b5d948cb34543e3881a96c730054172</t>
   </si>
   <si>
     <t>df_centrifuge_TG_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>52496c59ef184a7d968738e3d9bd30f2</t>
-  </si>
-  <si>
-    <t>f5b3a1b1f5264f51ba76bd940b252f37</t>
-  </si>
-  <si>
-    <t>dc0fd8d1aa3e4f89b03804d95d621fb5</t>
-  </si>
-  <si>
-    <t>4e39495f044046e09cc3752ede3ac80a</t>
+    <t>432a2e2ece89454283e9f5c7b31cac6d</t>
+  </si>
+  <si>
+    <t>499a4b6ebda24d9ab29dd6845b69db9d</t>
+  </si>
+  <si>
+    <t>cedecf3bbe2f4e4ea3d3bdf9b28605b3</t>
+  </si>
+  <si>
+    <t>7875fbe539024de1884d25f39ad3cf8a</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar de Olaroz</t>
@@ -1915,28 +1915,28 @@
     <t>df_centrifuge_general_1_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>8b98f306fb514ae6a81c16d5f98ace5a</t>
+    <t>9e68ddc4a3ac46438df62b56fc0423aa</t>
   </si>
   <si>
     <t>df_centrifuge_general_1_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>035ce47e0a8a42bd9acbacac927b2ffb</t>
-  </si>
-  <si>
-    <t>5746f9b50f844947b98ce88f6512bc93</t>
+    <t>a222385bb5fd43ad87eb8c19cfa85574</t>
+  </si>
+  <si>
+    <t>e4ec9d26c80c4d92990636d2bccd6ec3</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Silver Peak</t>
   </si>
   <si>
-    <t>8aa1e99e40d64bfe9f3fd78521e92f95</t>
+    <t>e585f7747c5347519243a20032e232af</t>
   </si>
   <si>
     <t>df_centrifuge_general_1_Zhabuye</t>
   </si>
   <si>
-    <t>e15b0aa3139e4039bcf6d5b64e213d5e</t>
+    <t>25962ed9706f40dc94804be9edfa5640</t>
   </si>
   <si>
     <t>df_washing_general_Zhabuye</t>
@@ -1948,7 +1948,7 @@
     <t>df_centrifuge_general_2_Salar de Olaroz</t>
   </si>
   <si>
-    <t>6a98412c8fbe490aa8ffc082dfa0a888</t>
+    <t>90c895b38c494ae88cf6bcb7fb669066</t>
   </si>
   <si>
     <t>df_centrifuge_general_2</t>
@@ -1960,7 +1960,7 @@
     <t>df_centrifuge_general_2_Silver Peak</t>
   </si>
   <si>
-    <t>a42f55c91bff40629cf69184cbcf0a56</t>
+    <t>0c9d544356f84e24ad3b72d97afa7e8f</t>
   </si>
   <si>
     <t>df_dissolution_Silver Peak</t>
@@ -1969,7 +1969,7 @@
     <t>df_centrifuge_general_2_Zhabuye</t>
   </si>
   <si>
-    <t>154cb36271cb42d78847ccfb2505a55e</t>
+    <t>f2f29f5464184fae90dbb9ccc99e6b20</t>
   </si>
   <si>
     <t>df_dissolution_Zhabuye</t>
@@ -1978,70 +1978,70 @@
     <t>df_centrifuge_purification_quicklime_East Taijinar</t>
   </si>
   <si>
-    <t>43ff7d4233634e71aef96f7149f5e940</t>
+    <t>243a0adba0fd4c90aded1dc6dde2c80b</t>
   </si>
   <si>
     <t>df_centrifuge_purification_quicklime_Maricunga</t>
   </si>
   <si>
-    <t>026c2f6395de4e90951bbbeea2cb3d11</t>
-  </si>
-  <si>
-    <t>b01e407a158a4d0785e806f366f67b04</t>
+    <t>13561aafc60d4c9c801bcbe9d339407a</t>
+  </si>
+  <si>
+    <t>9c4b1733750e4099b7da5792b3492f0d</t>
   </si>
   <si>
     <t>df_centrifuge_purification_quicklime_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>82021a9bc1e84d07a5fb4e8db1d014e7</t>
+    <t>7394467964d54e98a16ba93bb17a23a7</t>
   </si>
   <si>
     <t>df_centrifuge_purification_quicklime_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>1c4a09f724d14f169d8d2a93831cff76</t>
+    <t>701318181fad4a1eade27e9e060d96da</t>
   </si>
   <si>
     <t>df_centrifuge_purification_quicklime_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>8a43484ef30240c8b372b558a0aefcdd</t>
-  </si>
-  <si>
-    <t>05c5c89d9d2745f2a4ecddcfcd5dbbef</t>
+    <t>ea483f11aeee47a2ae5c19565442080c</t>
+  </si>
+  <si>
+    <t>178d37e4213643a9b2af1fd542af1822</t>
   </si>
   <si>
     <t>df_centrifuge_purification_sodaash_Sal de Vida</t>
   </si>
   <si>
-    <t>b18d1be6fef34f64b3e46fcd88dc8f03</t>
-  </si>
-  <si>
-    <t>f1587932a1284500878aab476ddd2b58</t>
-  </si>
-  <si>
-    <t>8b24a9bcfb5b4e16b22091fc8aff17f8</t>
+    <t>5c40b3b6893d40a59fed4ee626480c7f</t>
+  </si>
+  <si>
+    <t>38e360b74b6c45dc8053ac8c2256f04c</t>
+  </si>
+  <si>
+    <t>1e9a1cdf434c4a6bb8dabb79902f629e</t>
   </si>
   <si>
     <t>df_centrifuge_purification_sodaash_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>80fd8b7e47774b358e91ef427dfa9814</t>
+    <t>7a4ab80e9cb946d0a1931c80087e11f1</t>
   </si>
   <si>
     <t>df_centrifuge_purification_sodaash_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>2a50c5c7eef94ecdaf44f09942f6012d</t>
-  </si>
-  <si>
-    <t>01abfbd4e01b49218ef23ac05aa1b3b5</t>
+    <t>02423231b1244323835d2fece3268b1b</t>
+  </si>
+  <si>
+    <t>2e5cf1cdc49b48d581e11f8850513d47</t>
   </si>
   <si>
     <t>df_centrifuge_wash_Chaerhan</t>
   </si>
   <si>
-    <t>213febced79043b187f2fd4ae8108206</t>
+    <t>d6a2cadc5e594458bf7fa109ae763d68</t>
   </si>
   <si>
     <t>df_centrifuge_wash</t>
@@ -2056,7 +2056,7 @@
     <t>df_centrifuge_wash_East Taijinar</t>
   </si>
   <si>
-    <t>76027601817148db800c59b091366c9c</t>
+    <t>20b88acd4811455a9f13c384fac94d53</t>
   </si>
   <si>
     <t>df_washing_BG_East Taijinar</t>
@@ -2065,7 +2065,7 @@
     <t>df_centrifuge_wash_Fenix</t>
   </si>
   <si>
-    <t>cc3eba439f4a44d088475c0423be9101</t>
+    <t>86633ab51e5d4fbc88c9027cc3907eef</t>
   </si>
   <si>
     <t>df_washing_BG_Fenix</t>
@@ -2074,7 +2074,7 @@
     <t>df_centrifuge_wash_Kachi</t>
   </si>
   <si>
-    <t>b6f43e3553434e8ebb667276aaedb087</t>
+    <t>e5b57c65b2c248a1bc9a399ca91ac031</t>
   </si>
   <si>
     <t>df_washing_BG_Kachi</t>
@@ -2083,7 +2083,7 @@
     <t>df_centrifuge_wash_Lakkor Tso</t>
   </si>
   <si>
-    <t>d9804de0667c43578e08b8a031e784a5</t>
+    <t>13eb746b2a5043c8aad03b040f324e27</t>
   </si>
   <si>
     <t>df_washing_BG_Lakkor Tso</t>
@@ -2092,7 +2092,7 @@
     <t>df_centrifuge_wash_Maricunga</t>
   </si>
   <si>
-    <t>51fd7d7638af4221be397df9c2290c5f</t>
+    <t>4c94962e858e47b0aa18658727afc86b</t>
   </si>
   <si>
     <t>df_washing_BG_Maricunga</t>
@@ -2101,13 +2101,13 @@
     <t>df_centrifuge_wash_Pozuelos</t>
   </si>
   <si>
-    <t>375aaa385e4b4dd0a8a2d546c590d2b8</t>
+    <t>29f11de27fdb435981e88432b697a666</t>
   </si>
   <si>
     <t>df_centrifuge_wash_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>cc269d5f23d44e3ba4677fe482fee291</t>
+    <t>3097cffd563e4c9cad3ec7d2ad3c1f96</t>
   </si>
   <si>
     <t>df_washing_BG_Qinghai Yiliping</t>
@@ -2116,13 +2116,13 @@
     <t>df_centrifuge_wash_Sal de Vida</t>
   </si>
   <si>
-    <t>3eafa1c4a093409d94e05f307cf3f1b4</t>
+    <t>65d779b061d14268b8076e4c04b53ace</t>
   </si>
   <si>
     <t>df_centrifuge_wash_Sal de los Angeles</t>
   </si>
   <si>
-    <t>dcbefbc9314342cab579d356dd6c4f7e</t>
+    <t>c9e0f22b02d9470284696b1304a32365</t>
   </si>
   <si>
     <t>df_washing_BG_Sal de los Angeles</t>
@@ -2131,13 +2131,13 @@
     <t>df_centrifuge_wash_Salar de Arizaro</t>
   </si>
   <si>
-    <t>06586b9cc9104cb59b7d0b620867c78d</t>
+    <t>5f121cec4a154176b967c5fe11b27e9f</t>
   </si>
   <si>
     <t>df_centrifuge_wash_Salar de Atacama</t>
   </si>
   <si>
-    <t>f6b0b36cda4647c69a513563b6ed32f3</t>
+    <t>aa7b933022de482fb45efbdfba9e8d3c</t>
   </si>
   <si>
     <t>df_washing_BG_Salar de Atacama</t>
@@ -2146,7 +2146,7 @@
     <t>df_centrifuge_wash_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>43fea7687b3c440fae9c6ab6dbf675b4</t>
+    <t>599a53c64e2a476094bfa0924a42beb1</t>
   </si>
   <si>
     <t>df_washing_BG_Salar de Cauchari-Olaroz</t>
@@ -2155,7 +2155,7 @@
     <t>df_centrifuge_wash_Salar de Centenario</t>
   </si>
   <si>
-    <t>b658db3ec8794940b4c844cdf81b7b83</t>
+    <t>2bf2d60daaa849d29d405e6f101b41db</t>
   </si>
   <si>
     <t>df_washing_BG_Salar de Centenario</t>
@@ -2164,7 +2164,7 @@
     <t>df_centrifuge_wash_Salar de Olaroz</t>
   </si>
   <si>
-    <t>98cf8b4bf9e7442da8a0799074fe1585</t>
+    <t>8f0177673cbf4ac7a1e90691abc2f701</t>
   </si>
   <si>
     <t>df_washing_BG_Salar de Olaroz</t>
@@ -2173,19 +2173,19 @@
     <t>df_centrifuge_wash_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>1a6d775afabe4a6daaf8a9e53dc9474f</t>
+    <t>911442aaa71b4b10931533bf8f55b446</t>
   </si>
   <si>
     <t>df_centrifuge_wash_Salar de Tolillar</t>
   </si>
   <si>
-    <t>bd87e66d734f475d9191bc087956cb2b</t>
+    <t>e180e998e0414f3b81a8ad68295d1b2c</t>
   </si>
   <si>
     <t>df_centrifuge_wash_Salar de Uyuni</t>
   </si>
   <si>
-    <t>f6a8168a4abf4f818c45275ea75e9721</t>
+    <t>0eab2408a6874c809ac563dc467aff28</t>
   </si>
   <si>
     <t>df_washing_BG_Salar de Uyuni</t>
@@ -2194,13 +2194,13 @@
     <t>df_centrifuge_wash_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>56f9974267f64fc69fc5f08fdb598ffb</t>
+    <t>4c8596a260c2469a9bda5c90b1d31140</t>
   </si>
   <si>
     <t>df_centrifuge_wash_Salar del Rincon</t>
   </si>
   <si>
-    <t>3eea7dc7f59047e09a1c86932d4c2ec1</t>
+    <t>40b3664fcbba46d9ae17532c66703b2c</t>
   </si>
   <si>
     <t>df_washing_BG_Salar del Rincon</t>
@@ -2209,7 +2209,7 @@
     <t>df_centrifuge_wash_Silver Peak</t>
   </si>
   <si>
-    <t>e11b00e64aa4448c9be621de3f39abc8</t>
+    <t>9959a550541148df9e8fa352681fd186</t>
   </si>
   <si>
     <t>df_washing_BG_Silver Peak</t>
@@ -2218,7 +2218,7 @@
     <t>df_centrifuge_wash_Tres Quebradas</t>
   </si>
   <si>
-    <t>830fa0b34c1945b8a753e5c762fcfba8</t>
+    <t>52202d66e4ff48ffaa92128405da390b</t>
   </si>
   <si>
     <t>df_washing_BG_Tres Quebradas</t>
@@ -2227,7 +2227,7 @@
     <t>df_centrifuge_wash_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>b6007bd807c24dd0b1083dd4ace5b74b</t>
+    <t>9bec495af40a4e81b1a8441352041b9f</t>
   </si>
   <si>
     <t>df_washing_BG_Upper Rhine Graben</t>
@@ -2236,43 +2236,43 @@
     <t>df_centrifuge_wash_Zhabuye</t>
   </si>
   <si>
-    <t>0c88dcf7ccd84169b741df1566ad8e86</t>
+    <t>19af17b05a004b2b8d7396b506f8abbe</t>
   </si>
   <si>
     <t>df_washing_BG_Zhabuye</t>
   </si>
   <si>
-    <t>887d5690f0494661ae1f729e00ad318c</t>
+    <t>ba150beced1749a78a2295719aaf8d59</t>
   </si>
   <si>
     <t>df_washing_TG_Chaerhan</t>
   </si>
   <si>
-    <t>57591e232ac2490f90ccc7ee65a0fd06</t>
+    <t>6ce6bcfc5acb469eac0c67eddcd428eb</t>
   </si>
   <si>
     <t>df_washing_TG_East Taijinar</t>
   </si>
   <si>
-    <t>c291fd8762e14660a7fc96e6c0cdd227</t>
+    <t>f22b5b21ca3c451bb28a991df71fe2e4</t>
   </si>
   <si>
     <t>df_washing_TG_Fenix</t>
   </si>
   <si>
-    <t>5ccd4db93a784f77814d712105e9c028</t>
+    <t>d8c6340add99499796e35ad96df64bf2</t>
   </si>
   <si>
     <t>df_washing_TG_Kachi</t>
   </si>
   <si>
-    <t>a97a04d3038b4f2a96cbcb5bc9ab5f2a</t>
+    <t>14f07c1ae275424abebc44cb48b3fedc</t>
   </si>
   <si>
     <t>df_washing_TG_Lakkor Tso</t>
   </si>
   <si>
-    <t>cb7ac889ccc74522abdbffefbab65b31</t>
+    <t>d9cb6bee0d574c55b1dd7a3b0b5bf533</t>
   </si>
   <si>
     <t>df_washing_TG_Maricunga</t>
@@ -2281,10 +2281,10 @@
     <t>df_dissolution_Pozuelos</t>
   </si>
   <si>
-    <t>c799e4a7f5fe4217b565eed3481d4c18</t>
-  </si>
-  <si>
-    <t>f3d9818185634596886c461b34c795ec</t>
+    <t>1421997fa80b4178b4f80bcb2d88287c</t>
+  </si>
+  <si>
+    <t>77e1681effcf47a284930b356779f9b6</t>
   </si>
   <si>
     <t>df_washing_TG_Qinghai Yiliping</t>
@@ -2293,10 +2293,10 @@
     <t>df_dissolution_Sal de Vida</t>
   </si>
   <si>
-    <t>8f66f02f44fd43eca1af600f167c24be</t>
-  </si>
-  <si>
-    <t>55f59704aa2047428d21fb5b81b073e0</t>
+    <t>10293ecf2ee84318a724c2bb8e919b84</t>
+  </si>
+  <si>
+    <t>39462937d3ec466e8a9b763250747e9f</t>
   </si>
   <si>
     <t>df_washing_TG_Sal de los Angeles</t>
@@ -2305,43 +2305,43 @@
     <t>df_dissolution_Salar de Arizaro</t>
   </si>
   <si>
-    <t>c39c468a5a61421ba1bdf68021dc9b61</t>
-  </si>
-  <si>
-    <t>10b786f9c7bc4e09a9ec4a6a3ea312e0</t>
+    <t>f50383d991fb4ec69bbb0d3b14aacd14</t>
+  </si>
+  <si>
+    <t>6c0511a810e34ba09b408c5d611384ef</t>
   </si>
   <si>
     <t>df_washing_TG_Salar de Atacama</t>
   </si>
   <si>
-    <t>488459bd1c0e499a99e362a6c1dcfe77</t>
+    <t>4f1be0d31e4b4febb52d012a2c3262f5</t>
   </si>
   <si>
     <t>df_washing_TG_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>a27a26c235554633a17815d5cb3bb10f</t>
+    <t>8216c534332f439183f89e49a4c79dd9</t>
   </si>
   <si>
     <t>df_washing_TG_Salar de Centenario</t>
   </si>
   <si>
-    <t>bef804ebfcdd49fcb02caf83aef213ce</t>
+    <t>3c6adf0dd3ab4ac58fb5267ee58f82b4</t>
   </si>
   <si>
     <t>df_dissolution_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>d5cded6b1d5c442cb8b86d32c0f97be9</t>
+    <t>1f04f808300a43f2b963af6bcf37d4d0</t>
   </si>
   <si>
     <t>df_dissolution_Salar de Tolillar</t>
   </si>
   <si>
-    <t>6cb9aae186014dcf972e5a3f8325dc62</t>
-  </si>
-  <si>
-    <t>0e85ea7fb6be42ce9079c5cbe9df0a74</t>
+    <t>c1013dae23d64193a5b23f1f5b7302c5</t>
+  </si>
+  <si>
+    <t>702cfaf472094269bae611dafb38c31b</t>
   </si>
   <si>
     <t>df_washing_TG_Salar de Uyuni</t>
@@ -2350,37 +2350,37 @@
     <t>df_dissolution_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>dbaa96b7b143410698c721205b391419</t>
-  </si>
-  <si>
-    <t>543d984fb92f41d9884fa2256d4d2a3f</t>
+    <t>e2abfc6cf7a04a55885cc888b46106f0</t>
+  </si>
+  <si>
+    <t>354f5d826fd94dffbdc0814ee0338d4a</t>
   </si>
   <si>
     <t>df_washing_TG_Salar del Rincon</t>
   </si>
   <si>
-    <t>4df84446943c46ed882956aae1045c76</t>
-  </si>
-  <si>
-    <t>2282c5742ad94d20b584bb27145e2024</t>
+    <t>628dff8ee1e94b04b2d0ecd6bacca586</t>
+  </si>
+  <si>
+    <t>7b7930c004ac4a368b12f19b2217db26</t>
   </si>
   <si>
     <t>df_washing_TG_Tres Quebradas</t>
   </si>
   <si>
-    <t>314cd5f8269e4cd29bdf00cc4cfe60db</t>
+    <t>e5aa03242b5c41e0af33afc31e75fe38</t>
   </si>
   <si>
     <t>df_washing_TG_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>1296e090b1a74a6aba2becc5861b7809</t>
+    <t>86c3aed015dd4898a669ebcb3c472abe</t>
   </si>
   <si>
     <t>df_electrodialysis_East Taijinar</t>
   </si>
   <si>
-    <t>ab56719e9ce2426fac71d9863516ea9b</t>
+    <t>4bedc5f59d494d30b20aaa509eb8aadf</t>
   </si>
   <si>
     <t>df_electrodialysis</t>
@@ -2389,7 +2389,7 @@
     <t>df_ion_exchange_L_East Taijinar</t>
   </si>
   <si>
-    <t>1630b629666140dcb2ed38eaa3f66797</t>
+    <t>91ff8dc4390e43caac5acf280fe09e72</t>
   </si>
   <si>
     <t>machine operation, diesel, &gt;= 74.57 kW, high load factor</t>
@@ -2410,103 +2410,103 @@
     <t>salt tailing from potash mine</t>
   </si>
   <si>
-    <t>0cd8f2e047bb47d9b7b33114aa5b93c9</t>
-  </si>
-  <si>
-    <t>944deb3785bd4162bc5a39843bd56547</t>
-  </si>
-  <si>
-    <t>7e5540752be34befa13a0969b8a003c0</t>
-  </si>
-  <si>
-    <t>b576a1680bf74604bc64abcf2015b343</t>
-  </si>
-  <si>
-    <t>2739d5b15e2047fd83053f29ce040897</t>
+    <t>9b6a81a6150d46b3bf2fe4afa6530067</t>
+  </si>
+  <si>
+    <t>25d83603791a4a6fbc3bca180b42fc0e</t>
+  </si>
+  <si>
+    <t>b659414ac397440a9ff6088dc1e710db</t>
+  </si>
+  <si>
+    <t>c4b069dd2bba4296a6a75b2cec91579b</t>
+  </si>
+  <si>
+    <t>cdaa55548e414220b8eac87803137778</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Pozuelos</t>
   </si>
   <si>
-    <t>6ea8606d352d4adc8943677a3355a28b</t>
-  </si>
-  <si>
-    <t>31eedc8e2ae24bf99fbcf51e4807e36d</t>
+    <t>169201200f7241a48483243cd4916feb</t>
+  </si>
+  <si>
+    <t>282b0645177044e0a73ec830584a686c</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Sal de Vida</t>
   </si>
   <si>
-    <t>74f4e4f2d87548c7aa706a19051c4440</t>
-  </si>
-  <si>
-    <t>89c51a33e35e4a898e916535f9fcd3b5</t>
+    <t>4fedb253917d4fa6a262ef0a1f34bf2b</t>
+  </si>
+  <si>
+    <t>3c5ff856e6f849a590f7dca96a7e02e7</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar de Arizaro</t>
   </si>
   <si>
-    <t>9d8946222f4a418aa07552281a07a1e6</t>
+    <t>d39be5b3c8a74af382facc53cdb18c40</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar de Atacama</t>
   </si>
   <si>
-    <t>fdcb9381867049f3af6e3ee937f7b638</t>
-  </si>
-  <si>
-    <t>7ace368baff745e397cf5185f3d2f182</t>
-  </si>
-  <si>
-    <t>bcd238e473344a1dbe46febcdd90fdee</t>
-  </si>
-  <si>
-    <t>9980f26e81db40aeaef15164399f07db</t>
+    <t>0cf8c18e297442dfb2e27df17d721fab</t>
+  </si>
+  <si>
+    <t>b2b6fd24ca984431be5b25a69cfe74c9</t>
+  </si>
+  <si>
+    <t>142e6da0611f4f1380911cb9a839ea12</t>
+  </si>
+  <si>
+    <t>c235a347c7f54c6188b73fe041f66246</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>8d062b27e4c746c0b308e18c91e35cb7</t>
+    <t>f1093b689e444def97a7e5a3249a01a3</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar de Tolillar</t>
   </si>
   <si>
-    <t>2ab9003059da4177a6678ca25b42593c</t>
-  </si>
-  <si>
-    <t>2a86aaa1217c4e78bc8ce30cc7faa460</t>
+    <t>48376a62db9d4fb29b4d14b7758c214a</t>
+  </si>
+  <si>
+    <t>0275e1db825e4680bd4fe63b6f204c6d</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>536c52e5e0484630bfe1469cbd80d7c7</t>
-  </si>
-  <si>
-    <t>6e41d71ba6aa43a284594cdf819c646d</t>
-  </si>
-  <si>
-    <t>67c717ec95ce4ccebffb03d9c412f8f3</t>
+    <t>a9c0c128846c402fbe841648dd05530a</t>
+  </si>
+  <si>
+    <t>f3544b1c4a274ae98e825a63e07eba0b</t>
+  </si>
+  <si>
+    <t>acd27e43189c4c5285175b36e8abba74</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Tres Quebradas</t>
   </si>
   <si>
-    <t>127c217599b842af97ed10e6f1d10f10</t>
+    <t>999038035a0f4be0bf0bf7dd675726a3</t>
   </si>
   <si>
     <t>df_evaporation_ponds_Zhabuye</t>
   </si>
   <si>
-    <t>00cf4c1ff1064051b709721a9d1d025c</t>
+    <t>2b2ec683223b48c0a29c785782edbf20</t>
   </si>
   <si>
     <t>df_grinding_Zhabuye</t>
   </si>
   <si>
-    <t>334df311abd447bda5a8f7e5ed784ab0</t>
+    <t>c45135df55ff45e09b9f72a5039181af</t>
   </si>
   <si>
     <t>df_grinding</t>
@@ -2518,7 +2518,7 @@
     <t>df_ion_exchange_H_2_Salar de Olaroz</t>
   </si>
   <si>
-    <t>2b07600eb06044b98cf99b312bf6f647</t>
+    <t>3ca0ef7ead604cd6821c0fb211f04430</t>
   </si>
   <si>
     <t>df_ion_exchange_H_2</t>
@@ -2539,7 +2539,7 @@
     <t>df_ion_exchange_H_2_Silver Peak</t>
   </si>
   <si>
-    <t>3d31621e4b624cd2b881c739234dda8e</t>
+    <t>78382b40943a407dbdc55880c6171670</t>
   </si>
   <si>
     <t>df_ion_exchange_H_Silver Peak</t>
@@ -2548,61 +2548,61 @@
     <t>df_ion_exchange_H_2_Zhabuye</t>
   </si>
   <si>
-    <t>73dae37a5e37402ca1cdb9aa5a4437e7</t>
+    <t>3649847d130c41c9982f6d844a34efbe</t>
   </si>
   <si>
     <t>df_ion_exchange_H_Zhabuye</t>
   </si>
   <si>
-    <t>4bb7f7889bda4f49bca4315061b55f6e</t>
+    <t>b462c4e3256a42cf8ba92f7d5dd628f7</t>
   </si>
   <si>
     <t>df_ion_exchange_H_Sal de Vida</t>
   </si>
   <si>
-    <t>17a4237643e0439bbfcf14eb9be081ba</t>
+    <t>c25ab22bf95d463484580c9e3531af15</t>
   </si>
   <si>
     <t>df_ion_exchange_H_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>8eed0eb986f24faab796721ac659172e</t>
+    <t>b11ee1437daa43d38b8ab869e3392b48</t>
   </si>
   <si>
     <t>df_sulfate_removal_calciumchloride_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>645c2e19498745768469793934060098</t>
+    <t>dc000c884aa145fa802256ed7f0a2375</t>
   </si>
   <si>
     <t>df_ion_exchange_H_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>37f5774e9907424da990a2973c44d7ca</t>
-  </si>
-  <si>
-    <t>6ceb710d33c944ea879e18716e3699cd</t>
-  </si>
-  <si>
-    <t>31f910975a3f42da9ded8c77578175bc</t>
+    <t>0d949540de88461aa9ba7f13d3cb6d68</t>
+  </si>
+  <si>
+    <t>d2faf9e019d3467da13d449bc21eacb5</t>
+  </si>
+  <si>
+    <t>18578c874af346d9b5ec213c406b68c4</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Chaerhan</t>
   </si>
   <si>
-    <t>7791b57a83064ccc8da5cbbb04713db8</t>
-  </si>
-  <si>
-    <t>f886e6ba028347929525ff57d78db0c4</t>
-  </si>
-  <si>
-    <t>aa7512a8c5bb44c39591542ab36669db</t>
+    <t>477ffb8563f444d5a6e5d43e11984399</t>
+  </si>
+  <si>
+    <t>aa294bace125404e9d64b11b1776b4e6</t>
+  </si>
+  <si>
+    <t>2cacde18df404ed6a855680325d618c4</t>
   </si>
   <si>
     <t>df_triple_evaporator_Fenix</t>
   </si>
   <si>
-    <t>78ecaf74f01d45d896236fa3979068d8</t>
+    <t>dec36ec806424e5bbad6086c89231040</t>
   </si>
   <si>
     <t>df_triple_evaporator_Kachi</t>
@@ -2611,22 +2611,22 @@
     <t>df_ion_exchange_L_Lakkor Tso</t>
   </si>
   <si>
-    <t>8490af5196b4482fb7729a8c3870e459</t>
+    <t>8f5af0058e3c4ee0b72522cb280dcb89</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Pozuelos</t>
   </si>
   <si>
-    <t>254aa76ab94742b0969694f9d9d2be65</t>
+    <t>1c5856e4fc554e60a9b73822a37a9758</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>7af1127855d04aeebb9ff46e9d2aa10d</t>
-  </si>
-  <si>
-    <t>f06eff3a69a84a6ea79f6dc878c603f4</t>
+    <t>fcb9496d15d641a1b5187333f6bcb4ee</t>
+  </si>
+  <si>
+    <t>8cd69c52e68b417981f638061ea8f654</t>
   </si>
   <si>
     <t>df_triple_evaporator_Sal de los Angeles</t>
@@ -2635,52 +2635,52 @@
     <t>df_ion_exchange_L_Salar de Arizaro</t>
   </si>
   <si>
-    <t>0f3d0f10bf1849a5bb07012bc6421561</t>
-  </si>
-  <si>
-    <t>2799e8890ea04fc78e225ea798e44b78</t>
+    <t>b2e8ec8f2b884392be9c457f8ac260c7</t>
+  </si>
+  <si>
+    <t>c9521d5ac73f47fa9c2b83fbfb471244</t>
   </si>
   <si>
     <t>df_triple_evaporator_Salar de Centenario</t>
   </si>
   <si>
-    <t>4adb1e20ea834d7aabff8861240e6e9e</t>
+    <t>e057486a961f497984beeb9f476b39cf</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Salar de Tolillar</t>
   </si>
   <si>
-    <t>1cda4656d6404b56bcf6bce8f2031de9</t>
-  </si>
-  <si>
-    <t>783b285977e647ac873a2f986e9c9eb7</t>
+    <t>99c0f2b7e9554b83971a6ded0d1997a1</t>
+  </si>
+  <si>
+    <t>b3caa422ecc444c9aca7bc706a99bdaa</t>
   </si>
   <si>
     <t>df_triple_evaporator_Salar de Uyuni</t>
   </si>
   <si>
-    <t>db5d4f2adff64d0283de9095f9683d52</t>
+    <t>e63380b85f734794a7dbb9c4d0f317f7</t>
   </si>
   <si>
     <t>df_triple_evaporator_Salar del Rincon</t>
   </si>
   <si>
-    <t>fe5920cae1ae4dfb9b341caa9a4d3d44</t>
+    <t>30d447e98ec643519f3044f5960e67f8</t>
   </si>
   <si>
     <t>df_ion_exchange_L_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>a9c729b9ed314b2ea01b7c029531d463</t>
-  </si>
-  <si>
-    <t>95dc5f2996e5426a84398c7e7e9fe84c</t>
+    <t>5eca588d523b49a898b611c09e2efa13</t>
+  </si>
+  <si>
+    <t>d14d02b9a1684914a9b60ff2bf5fa1a9</t>
   </si>
   <si>
     <t>df_nanofiltration_Chaerhan</t>
   </si>
   <si>
-    <t>6af36d288b1049ecbf44745415aabf1b</t>
+    <t>4b202f8f45b948c0a327325929ef39a4</t>
   </si>
   <si>
     <t>df_nanofiltration</t>
@@ -2689,175 +2689,175 @@
     <t>df_nanofiltration_Lakkor Tso</t>
   </si>
   <si>
-    <t>d1c863c39fa0416d9b354fa5204779f4</t>
+    <t>89fc7b2dfc8e4915abac3e6c3706f169</t>
   </si>
   <si>
     <t>df_nanofiltration_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>a94648330df047bf9729cc437479c8da</t>
-  </si>
-  <si>
-    <t>793a8b602453476286760c79daed4758</t>
-  </si>
-  <si>
-    <t>ae2ca868c2864b979e08aa4dee4ee1a1</t>
-  </si>
-  <si>
-    <t>6aeab942f5c1463e991851a0cb11e16e</t>
-  </si>
-  <si>
-    <t>6484357b94d640b2b43321e51485f25c</t>
+    <t>47001bc487454ec4918186c8c4b03901</t>
+  </si>
+  <si>
+    <t>d5f48c169ba34cc7aaaa18fa89f4f1ce</t>
+  </si>
+  <si>
+    <t>2762a0b081584e40b0ae665c82344d0c</t>
+  </si>
+  <si>
+    <t>7f8ec30470944ca891ee47991f95d157</t>
+  </si>
+  <si>
+    <t>51a19666049844deada888ef83b4bdb5</t>
   </si>
   <si>
     <t>df_reverse_osmosis_Upper Rhine Graben</t>
   </si>
   <si>
-    <t>d8933cb87fef4f318bde41c1919878e2</t>
+    <t>0fe9d5a96236432fabd99905aff920a2</t>
   </si>
   <si>
     <t>df_rotary_dryer_Chaerhan</t>
   </si>
   <si>
-    <t>90e7005f3cdf4d1bbd472aeb38cbe316</t>
+    <t>ea58bf5b548a47b3bdee2a530c27e079</t>
   </si>
   <si>
     <t>df_rotary_dryer_East Taijinar</t>
   </si>
   <si>
-    <t>08dfe84fd218473d877efd10d12dba83</t>
+    <t>1aef0eb72a3e4a0790f12904262261e4</t>
   </si>
   <si>
     <t>df_rotary_dryer_Fenix</t>
   </si>
   <si>
-    <t>b818da93eb54469c9ce202b06a06987e</t>
+    <t>5ecdbc6effb54aab9daf309268f71f2a</t>
   </si>
   <si>
     <t>df_rotary_dryer_Kachi</t>
   </si>
   <si>
-    <t>73d71954f30d4793845cab178d12af6f</t>
+    <t>03a78db8c285484794b03ae55a0ba6a5</t>
   </si>
   <si>
     <t>df_rotary_dryer_Lakkor Tso</t>
   </si>
   <si>
-    <t>175fdd936f4240f289191929249661c2</t>
+    <t>4d758e32588d4a4582d6f612fd72b9d6</t>
   </si>
   <si>
     <t>df_rotary_dryer_Maricunga</t>
   </si>
   <si>
-    <t>470b8189ac5c471f973dee37f6116f29</t>
+    <t>68639d543eaf4aecb9c4aa4fd313f93b</t>
   </si>
   <si>
     <t>df_rotary_dryer_Pozuelos</t>
   </si>
   <si>
-    <t>17b41afd491c46a08991733c9bd5c204</t>
+    <t>569b4210b27b4efbb056973a0832e5ae</t>
   </si>
   <si>
     <t>df_rotary_dryer_Qinghai Yiliping</t>
   </si>
   <si>
-    <t>1263dab60ba641849de1ea60f27a90bf</t>
+    <t>721225135ab74fd9b3192221722d2104</t>
   </si>
   <si>
     <t>df_rotary_dryer_Sal de Vida</t>
   </si>
   <si>
-    <t>e1f78ed6ca1c40a2b5fdd316ac67914a</t>
+    <t>b37d8aa5a2c54c76968b3706cdede3d5</t>
   </si>
   <si>
     <t>df_rotary_dryer_Sal de los Angeles</t>
   </si>
   <si>
-    <t>7ad32b92c84b4f0e8c7f84f5ce7f89cf</t>
+    <t>61ab916f33e3457a9e36aae11b212149</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar de Arizaro</t>
   </si>
   <si>
-    <t>5fc6b16ef2d5470bb0f81b3d05b8bd11</t>
+    <t>74eae9187cd34c82bc7d03133217343b</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar de Atacama</t>
   </si>
   <si>
-    <t>d0df62834ccc4b0781c5151ecbe3a705</t>
+    <t>2dcd2b1dfc5c491ba02a9af64adbef31</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>cf5bc117caf740a4a54c5a6c1b5903ab</t>
+    <t>9dbd98540c1c427d83296e27631a39ad</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar de Centenario</t>
   </si>
   <si>
-    <t>e44dbf85ac4048aaa3666781599c9209</t>
+    <t>1820176549dd4806a533d3bce89b83dc</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar de Olaroz</t>
   </si>
   <si>
-    <t>1aa1046a3fc24b1bbc3757d51b7d7b07</t>
+    <t>642672a545e848e3898cad7fd696dbe7</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>e284c4cdae3c4a499aaa22120fc5d05c</t>
+    <t>1eaa0da9261b4361ad6041fd9e6a1338</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar de Tolillar</t>
   </si>
   <si>
-    <t>d897922aa8b54ed795e7567ca5be4478</t>
+    <t>94b35de510084b06a6f722b51f558e40</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar de Uyuni</t>
   </si>
   <si>
-    <t>ea38658e7001467aa83b1c9555878624</t>
+    <t>be7c0525923c48938fb76ff664bc2dae</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>1a838e0e320144cc84a46c7d695e1d6c</t>
+    <t>c08aede2cfb4420c8b11b06285bf46be</t>
   </si>
   <si>
     <t>df_rotary_dryer_Salar del Rincon</t>
   </si>
   <si>
-    <t>4453d93c3ecb4979982200c07b80165d</t>
+    <t>3c780832780046a69296c4a8a998f5b7</t>
   </si>
   <si>
     <t>df_rotary_dryer_Silver Peak</t>
   </si>
   <si>
-    <t>37227d06d9b949a1b84580cec6cb7185</t>
+    <t>eccb7454ad4a485884b3cce9cffe1b42</t>
   </si>
   <si>
     <t>df_rotary_dryer_Tres Quebradas</t>
   </si>
   <si>
-    <t>e977cf9a73cf47169a24b90885c9f194</t>
-  </si>
-  <si>
-    <t>1480ca5d4edf4497bad0d4f84213d687</t>
+    <t>79e09ad4399e42aa802b13970858e0ac</t>
+  </si>
+  <si>
+    <t>5b579450393247b2993d024ad6e1fa41</t>
   </si>
   <si>
     <t>df_rotary_dryer_Zhabuye</t>
   </si>
   <si>
-    <t>e82bf730a0944dd1b02c116faf1c99e2</t>
-  </si>
-  <si>
-    <t>1f1b7c4d01ec4c9896827669777780cd</t>
+    <t>f76b66891bac4f04a7e3c2f7eb6de8c4</t>
+  </si>
+  <si>
+    <t>ed4a848544bb4e5eb48b02857634c4dc</t>
   </si>
   <si>
     <t>market for calcium chloride</t>
@@ -2866,10 +2866,10 @@
     <t>calcium chloride</t>
   </si>
   <si>
-    <t>2a5eea7abb2b405e96c2537487018f1d</t>
-  </si>
-  <si>
-    <t>5de8cfded2ee4822a8bafdf2e1f10072</t>
+    <t>41f464ed3d1047bbb723d4726258c862</t>
+  </si>
+  <si>
+    <t>14b80bfcfd134661b8bcf743823a178c</t>
   </si>
   <si>
     <t>transport, freight, lorry &gt;32 metric ton, EURO3</t>
@@ -2878,13 +2878,13 @@
     <t>ton kilometer</t>
   </si>
   <si>
-    <t>51959075ce4d4d9ca718ca7233168b3f</t>
-  </si>
-  <si>
-    <t>e5d574092f764fb98b806434dd28d85e</t>
-  </si>
-  <si>
-    <t>f290a7aae46f40aab806c91ddb11e1ec</t>
+    <t>2916d78f73bb477e9b6c80d385961ce3</t>
+  </si>
+  <si>
+    <t>4d7054b4450f4d5287df30136027a5d6</t>
+  </si>
+  <si>
+    <t>ae7939cfb79c4a71b1f91796a6d28064</t>
   </si>
   <si>
     <t>market for steam, in chemical industry</t>
@@ -2893,229 +2893,229 @@
     <t>steam, in chemical industry</t>
   </si>
   <si>
-    <t>6beed994ed7b4ae2ae9baebdd16009a0</t>
+    <t>7dd2dbc26b554ccca39cd70ce5587638</t>
   </si>
   <si>
     <t>df_triple_evaporator_Pozuelos</t>
   </si>
   <si>
-    <t>f8752f7b58004019be41be0471d628fa</t>
-  </si>
-  <si>
-    <t>61e8b227e9814549833987d2e8238a1d</t>
+    <t>f1b375093e90404a87102d7715c60a66</t>
+  </si>
+  <si>
+    <t>630c7af835934681b1881a3b8ce8f417</t>
   </si>
   <si>
     <t>df_triple_evaporator_Salar de Arizaro</t>
   </si>
   <si>
-    <t>9c44a6839021460b823f50e8a4e2f89c</t>
-  </si>
-  <si>
-    <t>d8f513234ef047fcb8fb90bd28d530a2</t>
-  </si>
-  <si>
-    <t>1e5d23dd1c504f3987bbb8e82ed556e1</t>
+    <t>f6f4937c04f5403e9be7f88ef00aa045</t>
+  </si>
+  <si>
+    <t>0bac9237fe8b46e9a5ffd3b5b9224bf6</t>
+  </si>
+  <si>
+    <t>cc0f8646ab4a44d3b09224da160cb8bf</t>
   </si>
   <si>
     <t>df_triple_evaporator_Salar de Tolillar</t>
   </si>
   <si>
-    <t>bba85d59cdc44ae3bced00c99cbbc2b1</t>
-  </si>
-  <si>
-    <t>1c7b2354a1134da490ee6f27104851d7</t>
-  </si>
-  <si>
-    <t>3ab22029931c49a0b106ff87dfc9f11e</t>
-  </si>
-  <si>
-    <t>d923f2d733dd4db3a8afb252aeeec60d</t>
-  </si>
-  <si>
-    <t>28e240dcee744c32a16b8807aa4f80de</t>
-  </si>
-  <si>
-    <t>e28d1e1b0126461d8cd038535ef1ac0d</t>
-  </si>
-  <si>
-    <t>06b766dfdc144ce4a19802d2415d6fad</t>
-  </si>
-  <si>
-    <t>5fb16d47486648cda771197901b3d766</t>
-  </si>
-  <si>
-    <t>b7d7dcd380764e7ba963598761707e01</t>
-  </si>
-  <si>
-    <t>b6499b9f11a74ac89ec05bfb4394422b</t>
+    <t>025989a93c3b4963982990f3da4619c2</t>
+  </si>
+  <si>
+    <t>04af997c441b46b0adf0f69166a9965c</t>
+  </si>
+  <si>
+    <t>fddad640ac5e40ba9926bb933cb2873f</t>
+  </si>
+  <si>
+    <t>f8d7a320db69419ea80dfc66fa8877db</t>
+  </si>
+  <si>
+    <t>41de524780894eb9b6631c5cbbe78074</t>
+  </si>
+  <si>
+    <t>6a4bfe77e58948b1af831f80739a1cad</t>
+  </si>
+  <si>
+    <t>e220ea5566f741619329d7d8aad7403e</t>
+  </si>
+  <si>
+    <t>bc074dba60344813b29961bceded7229</t>
+  </si>
+  <si>
+    <t>2fb182d799bf49919cf78823ee2ed30c</t>
+  </si>
+  <si>
+    <t>8bba0b3c50634b23a7fa60f202c72a60</t>
   </si>
   <si>
     <t>df_washing_BG_Pozuelos</t>
   </si>
   <si>
-    <t>af53fdf2c8684c119e849df435d94520</t>
-  </si>
-  <si>
-    <t>373bf21543434ed3a619ea356ab94b1c</t>
+    <t>dcb1e005c94c4939a88b346d1367f766</t>
+  </si>
+  <si>
+    <t>474ceb21a67440d1bcc800120212ea1a</t>
   </si>
   <si>
     <t>df_washing_BG_Sal de Vida</t>
   </si>
   <si>
-    <t>8e618e884f344ed98d07b36387a1dc2e</t>
-  </si>
-  <si>
-    <t>405c356843cf419c8331ea433d0431c3</t>
+    <t>6a699850f3014ce0a7cdd06d68d2bde8</t>
+  </si>
+  <si>
+    <t>ea73e8b743d7438b94c435b34cce3349</t>
   </si>
   <si>
     <t>df_washing_BG_Salar de Arizaro</t>
   </si>
   <si>
-    <t>3f7f24aaa4084cd9a860618dc096ff63</t>
-  </si>
-  <si>
-    <t>e50ff332a1a94f17a85b2ad2014c43c7</t>
-  </si>
-  <si>
-    <t>d296095a5fec4d12a4d896b2aee0fb62</t>
-  </si>
-  <si>
-    <t>405baab4d8bf4b32bde2b059b72cc50d</t>
-  </si>
-  <si>
-    <t>5931960f67fa405885434a01abd9550a</t>
+    <t>4f5da8f1e294412899dda0b31ec80fd9</t>
+  </si>
+  <si>
+    <t>618901ba6583480aa83c8986d9b64eb6</t>
+  </si>
+  <si>
+    <t>1545fd076d564f08af5b26315caa26b7</t>
+  </si>
+  <si>
+    <t>b676f2453ac44aefbeb40418b54b2cb4</t>
+  </si>
+  <si>
+    <t>786ae70eb455478e93cf115f92753ca6</t>
   </si>
   <si>
     <t>df_washing_BG_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>83871570e5f44a94a6e5ef35eb2d834a</t>
+    <t>e38cec8b4ef44970b09e6ee97efe9977</t>
   </si>
   <si>
     <t>df_washing_BG_Salar de Tolillar</t>
   </si>
   <si>
-    <t>3a9efd5b30fa47e0a62906716da3a907</t>
-  </si>
-  <si>
-    <t>e5ad4474441347fd8b344dabee568f7d</t>
+    <t>487a0c1823294722bc3b36825cca640d</t>
+  </si>
+  <si>
+    <t>d526dcb304cf44b99104555ae01f8e65</t>
   </si>
   <si>
     <t>df_washing_BG_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>0cf83bc08bc84325886abe591630d4fa</t>
-  </si>
-  <si>
-    <t>7243067775bf4177a46423a6a3215c4d</t>
-  </si>
-  <si>
-    <t>f6491cf62d4c4a5abfc567ab702a8df6</t>
-  </si>
-  <si>
-    <t>3a1821e96eee451098138dbb192cad23</t>
-  </si>
-  <si>
-    <t>4eeaf18463cc41b88107cccca7b202f4</t>
-  </si>
-  <si>
-    <t>1b8f5898f5804f8fb89c317e5ec5c60b</t>
-  </si>
-  <si>
-    <t>4a8f17b530f440b2a9f1f0bef7868c00</t>
-  </si>
-  <si>
-    <t>18b57cf1dc314ab780c287cf3b4dcdea</t>
-  </si>
-  <si>
-    <t>ae663fbd10bc4fea977aff6ab369440c</t>
-  </si>
-  <si>
-    <t>4f25fe3f0cf347bbacdeac311c61cb3a</t>
-  </si>
-  <si>
-    <t>6a0dbd48a4944dac9d94a28a997ac8b6</t>
-  </si>
-  <si>
-    <t>211e09a66ecf4130a615424011c2cbd9</t>
+    <t>39bf3fda32364bb2b3c45c10c70114a4</t>
+  </si>
+  <si>
+    <t>0351d3171c1b4d409d0897dd1d7a931a</t>
+  </si>
+  <si>
+    <t>cbe646845bb8416a803d1469bdcfb3bd</t>
+  </si>
+  <si>
+    <t>d50c54863a3a46e5971f3ca12301e38b</t>
+  </si>
+  <si>
+    <t>789b148aedd64cfcabc9f1e8825395b0</t>
+  </si>
+  <si>
+    <t>9a74b3948d6c4de69ef7f99e07f45cb5</t>
+  </si>
+  <si>
+    <t>56399eb713be4323bc7ce08f5b3ce90a</t>
+  </si>
+  <si>
+    <t>f2e507ed5fef45fcb579a300ee4f87cc</t>
+  </si>
+  <si>
+    <t>3b0cfbbeece040ef9a7e5980a9551a43</t>
+  </si>
+  <si>
+    <t>13e3509b816e4e40ab2617e7d43cf85e</t>
+  </si>
+  <si>
+    <t>67a8a50506704ec589da7fe82ac42eca</t>
+  </si>
+  <si>
+    <t>78db50459dc948209565290910f971a8</t>
   </si>
   <si>
     <t>df_washing_TG_Pozuelos</t>
   </si>
   <si>
-    <t>85c00b8a472f40a0a068eb835e246f6d</t>
-  </si>
-  <si>
-    <t>bd146337747d4f9c90aeaa1174f56f6c</t>
+    <t>a4b5235772204552beef0f589ab416cf</t>
+  </si>
+  <si>
+    <t>f113e4b7f8354dcf85be563dee6ab4df</t>
   </si>
   <si>
     <t>df_washing_TG_Sal de Vida</t>
   </si>
   <si>
-    <t>d848fac0fd584a5ab8e9798cc96e4d57</t>
-  </si>
-  <si>
-    <t>3275d3e31bb44a779045bfb4c9d2e336</t>
+    <t>fa69bfe01ca04aa6a51836978dabc067</t>
+  </si>
+  <si>
+    <t>2148b61907b44895822da4a338bf7ea3</t>
   </si>
   <si>
     <t>df_washing_TG_Salar de Arizaro</t>
   </si>
   <si>
-    <t>08552858bbde4c109636fa878761bdb3</t>
-  </si>
-  <si>
-    <t>550df7d8bfa04928bffe402d2635e92e</t>
-  </si>
-  <si>
-    <t>a57f83dab7ec4315a105d1fa2b78a203</t>
-  </si>
-  <si>
-    <t>e7dd4d63633e4e2a966b1f4419c0c3f6</t>
-  </si>
-  <si>
-    <t>e90c308b1da44686ab8a093a93216839</t>
+    <t>eb2721d80dc64ef4a7015186713ca3a4</t>
+  </si>
+  <si>
+    <t>bc222c73afe946adbc2a8b257fde9f83</t>
+  </si>
+  <si>
+    <t>3b94ed8862b340c6b1ac4076651828f3</t>
+  </si>
+  <si>
+    <t>bfadaab6a548453ba5670615b20317e5</t>
+  </si>
+  <si>
+    <t>92f50324a78542d983c5dcd4016fbedd</t>
   </si>
   <si>
     <t>df_washing_TG_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>734d06a2a1024e4a86e2dee83d9460a4</t>
+    <t>1e786fc362494fa6b7c7620098236ae1</t>
   </si>
   <si>
     <t>df_washing_TG_Salar de Tolillar</t>
   </si>
   <si>
-    <t>e81e2d54cea34eef9a126b2b41c2194d</t>
-  </si>
-  <si>
-    <t>779d116f195f4900a75961927b48aa7c</t>
+    <t>e0a9caaf0b714421bc894159060d9cd3</t>
+  </si>
+  <si>
+    <t>e175c4100f724a8287e178d1d2503679</t>
   </si>
   <si>
     <t>df_washing_TG_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>0f164fad17ea4a61ad28bae10e7ffc9e</t>
-  </si>
-  <si>
-    <t>b99962d690c94b44b5f6d267f1751ef1</t>
-  </si>
-  <si>
-    <t>840861ae8586423098f15ce71265cf24</t>
-  </si>
-  <si>
-    <t>55513f92fd054322a6799194ff1c96c8</t>
-  </si>
-  <si>
-    <t>e8e1f0fab8184ab48e2b8d8df598ecec</t>
-  </si>
-  <si>
-    <t>2bec3a8fe3e54bc29be4d20ac95c0dd7</t>
+    <t>a61a04f11207453c9a9aff13f43ccd1c</t>
+  </si>
+  <si>
+    <t>906ef414ab8f48208765a88324349102</t>
+  </si>
+  <si>
+    <t>7abb958c2db4454e847568f214cc94ba</t>
+  </si>
+  <si>
+    <t>5fc1a4c43aae4a5280410b47c504025b</t>
+  </si>
+  <si>
+    <t>3635430ed4a149e9930f11cfdd746fd2</t>
+  </si>
+  <si>
+    <t>f212c9c0aee8446c8b88b00aa1f1c6b6</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Chaerhan</t>
   </si>
   <si>
-    <t>5a2bb09405ce4eee9b569ca3de2281a8</t>
+    <t>d499790a2ad449f4bc1c0bb28acd03bc</t>
   </si>
   <si>
     <t>database</t>
@@ -3145,337 +3145,337 @@
     <t>heat production, at heat pump 30kW, allocation exergy, East Taijinar</t>
   </si>
   <si>
-    <t>ef53fbf1169c4582bb7e4707a88dca05</t>
+    <t>259b399bd97c471cb99ac6faea8136b1</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Fenix</t>
   </si>
   <si>
-    <t>18ab38a755c1447bb30e992c4a99102f</t>
+    <t>fb77e71e84a142049fb798a5597f11c4</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Kachi</t>
   </si>
   <si>
-    <t>f46586c7946745ec967b125965122a6d</t>
+    <t>996b717bfc7d426b8bffbfc5e62b60a3</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Lakkor Tso</t>
   </si>
   <si>
-    <t>d00719a8dcc54000ad667283fac12e93</t>
+    <t>59842d2b88784ad199d917256b0f1ac8</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Maricunga</t>
   </si>
   <si>
-    <t>7e0660d3a8004f50b9033baf5f749892</t>
+    <t>361be9061fd04e6f83800706dc3950ac</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Pozuelos</t>
   </si>
   <si>
-    <t>50a34dc1c1354a07a0028db910091e66</t>
+    <t>8aaccbfde8b14e2bbb7657eecd0a582c</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Qinghai Yiliping</t>
   </si>
   <si>
-    <t>17c06fc550034c9bb234ed24964db5e7</t>
+    <t>81f7d866a8f5410c828c915811d04de8</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Sal de Vida</t>
   </si>
   <si>
-    <t>c06a7755ae5549cabf991ce1d77c2579</t>
+    <t>0f1c4eed38b241fa91d5d608e308cec6</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Sal de los Angeles</t>
   </si>
   <si>
-    <t>e2a55cef654c47eeab31c30c700465f4</t>
+    <t>bf19e636901c4f0eb0976ec498adf2ea</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar de Arizaro</t>
   </si>
   <si>
-    <t>cd87f252a1c848309bed0164330b53a0</t>
+    <t>84f9c5ca30a54938b26f8d5b13f54fb5</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar de Atacama</t>
   </si>
   <si>
-    <t>ed34010217924cc6bf232c03889b68cd</t>
+    <t>3d8125d185dc4ebfac68915a605080f7</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>b7ffa77556f447bab5d5e4a24fddf505</t>
+    <t>255113d331c9436aaca62410f895070d</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar de Centenario</t>
   </si>
   <si>
-    <t>39f4e32849bf4da899d9b0e2a431779a</t>
+    <t>6aca51a5b1a048b796b98f6d2ce4d2a1</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar de Olaroz</t>
   </si>
   <si>
-    <t>39914e9b20e549d6b18235c37b1337be</t>
+    <t>53d9b2715a2f4dea924aac739899e331</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>e46cb3020d04473595c352a6be74ef88</t>
+    <t>434f9e89509a4ef4b6ca5efcf686679b</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar de Tolillar</t>
   </si>
   <si>
-    <t>99be6d74e437448face6aa69a2ae49b5</t>
+    <t>70dfc531730343c18cf8f2e29cba57f6</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar de Uyuni</t>
   </si>
   <si>
-    <t>a0ad2875b1d44500bd63f4721b23bead</t>
+    <t>a88c129ee34d474b967f69eef1b56064</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>80e33164d76544a7bdf54dc6306793d6</t>
+    <t>d2a4f6c153094d85bd3a373bfe485c2e</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Salar del Rincon</t>
   </si>
   <si>
-    <t>633aa03289464613966012777345aada</t>
+    <t>712926350ea04ecfa4df490277238af7</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Silver Peak</t>
   </si>
   <si>
-    <t>7620f54c19f44f2aa9970c47f3af2fbb</t>
+    <t>634be80694c5414bbef5d753926add0f</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Tres Quebradas</t>
   </si>
   <si>
-    <t>e5ce9fb6128648fe84b5ae7049d41e70</t>
+    <t>a6ec70b88d634f52b022283232f82644</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Upper Rhine Graben</t>
   </si>
   <si>
-    <t>ed137b055c314a99b7fe7ff16df220a3</t>
+    <t>1afe5235b8354dafa40332d7d09c3e10</t>
   </si>
   <si>
     <t>heat production, at heat pump 30kW, allocation exergy, Zhabuye</t>
   </si>
   <si>
-    <t>b8656311eab2420194f06aa2df5b7bae</t>
+    <t>4bada575b0ff49d99031bcf1b3c60757</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Chaerhan</t>
   </si>
   <si>
-    <t>1808b6b30bef4b9bb2712a5c53275c43</t>
+    <t>501bb177844a4f709474775b9ed91ac7</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, East Taijinar</t>
   </si>
   <si>
-    <t>6c946bc1611845be8932d75e6de4b688</t>
+    <t>fcc8e7a1e1e7436488b29448676d84b6</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Fenix</t>
   </si>
   <si>
-    <t>54e7fab3ccd44eabbcf1d9735f780273</t>
+    <t>25e41f7cb371465ebb0ff97540bd5ee9</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Kachi</t>
   </si>
   <si>
-    <t>00a0f74ee3624f968b164416e9046558</t>
+    <t>eee3ccf3e9184cd48d77ce477a2ce302</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Lakkor Tso</t>
   </si>
   <si>
-    <t>eb16fef73c084f15919dbfcb050a9bcd</t>
+    <t>abe1caefdce64dc2ba574020222e580c</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Maricunga</t>
   </si>
   <si>
-    <t>865520064f0d492b8c5f5e693778c253</t>
+    <t>eb5a59d40fb446c4bffc157d29d98ca9</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Pozuelos</t>
   </si>
   <si>
-    <t>5a830fb12daa4d978690ace365a79862</t>
+    <t>2a88c89dd1a94e74971e51edf6cc1a9b</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Qinghai Yiliping</t>
   </si>
   <si>
-    <t>965361d5f6434dde89d5057865cc6590</t>
+    <t>c6172957161f48f0bd0a3914036d2e43</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Sal de Vida</t>
   </si>
   <si>
-    <t>817161df7a694f4a8a12e32bff4db0be</t>
+    <t>25c9b7a73793460fb019a4d4c752f7c0</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Sal de los Angeles</t>
   </si>
   <si>
-    <t>419bee3f289d46e39fc583fbe53440d6</t>
+    <t>0ab56a26fb2948e19b084a8edddaf6ba</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Salar de Arizaro</t>
   </si>
   <si>
-    <t>a835cd6bd8b04355b4a3b838ca4363e7</t>
+    <t>fd2582afee774e8bb96e272c5edb5fc0</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Salar de Atacama</t>
   </si>
   <si>
-    <t>8eafc25578c64305980fbbb1bcf6ba20</t>
+    <t>c75a0aa415d9433ab9c35f0f0eb13f51</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Salar de Cauchari-Olaroz</t>
   </si>
   <si>
-    <t>c71159a3d0fc49e781da6377c9b3acdd</t>
+    <t>c267a3a40e6d47b09ec8ecceece7ee68</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Salar de Centenario</t>
   </si>
   <si>
-    <t>4e1bd215b46445c0a4daa44529424dff</t>
+    <t>fd7b0871691e43ed844d13c2ad0b91b1</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Salar de Olaroz</t>
   </si>
   <si>
-    <t>e99685964d1c474e867c7f803568ff11</t>
+    <t>a2350b671ec940e6a5b4f1ab8350085a</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>ed2fd59a1ffe4eb58263da409b47a764</t>
+    <t>0a50d40788fe47468aa07245a36ab58f</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Salar de Tolillar</t>
   </si>
   <si>
-    <t>da3879a94be6407298346650e5c4c224</t>
+    <t>fe6493285ddf40ec8f049c004db0f99e</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Salar de Uyuni</t>
   </si>
   <si>
-    <t>ee1e050f4ec34f6dbeacaba9dbaa00c3</t>
+    <t>ad05a991a10e4253befa9e68956020ea</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>8c9d5eea18454224816be6af2e6044b0</t>
-  </si>
-  <si>
-    <t>0076d910a69a442d86afd4f1bc981e41</t>
+    <t>2dca35db848f482b895aa34dfb6668b4</t>
+  </si>
+  <si>
+    <t>76d78bfc0cd9437da373d3ac8ce22db7</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Silver Peak</t>
   </si>
   <si>
-    <t>9e04476cceee4ec19f0da13d9aef032f</t>
+    <t>cf9064c415574281866a969826d5488e</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Tres Quebradas</t>
   </si>
   <si>
-    <t>de37128425a94dd0b5f9de5a4e82d16c</t>
+    <t>707d8b607e634428adefd9f02096d895</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Upper Rhine Graben</t>
   </si>
   <si>
-    <t>bf790074beb9437693470fe8f5242a9e</t>
+    <t>99d161474c484d44a1590b4528f5a741</t>
   </si>
   <si>
     <t>heat production, industrial electric boiler, Zhabuye</t>
   </si>
   <si>
-    <t>87e35023b4124f3ca2cbe2ab910ec417</t>
-  </si>
-  <si>
-    <t>ef695e2580264e6394a3528f5be1ddc3</t>
+    <t>5209ca6ecbbf4710aa92513664a23e57</t>
+  </si>
+  <si>
+    <t>8d090b6070074a9f906698a688e113f7</t>
   </si>
   <si>
     <t>waste_liquid_Ari_Salar de Arizaro</t>
   </si>
   <si>
-    <t>292cad106b524e7fa28ba007a6e58760</t>
+    <t>f32f0bf4fc834c56aeb495adddf5c706</t>
   </si>
   <si>
     <t>waste_liquid_Ari</t>
   </si>
   <si>
-    <t>b3a64daa8bd1453f8db1e82c10486527</t>
-  </si>
-  <si>
-    <t>d81b46443d074693b1a6df6feb8e607c</t>
-  </si>
-  <si>
-    <t>be74b7d5ecf5456492cf5c7b1386ac23</t>
-  </si>
-  <si>
-    <t>5fde7470dc4141768b433969e556abe7</t>
-  </si>
-  <si>
-    <t>246c8ec99bf949ce80319072b1bf3ebc</t>
-  </si>
-  <si>
-    <t>880e6d590ae44c07ba8d7eb51baf2c23</t>
+    <t>92b7000819454b2180d6a249cb2dca84</t>
+  </si>
+  <si>
+    <t>c6e08cf5d5c94bfda5e33dd31e521cac</t>
+  </si>
+  <si>
+    <t>211d869c665b40e0a3a1bf1793b0455c</t>
+  </si>
+  <si>
+    <t>ada268e27b7542ffb93a2f4755b35eb6</t>
+  </si>
+  <si>
+    <t>e2d9b81a294d4d6688e7f2bcde760438</t>
+  </si>
+  <si>
+    <t>1fdf911a79a145cf930cd62194963603</t>
   </si>
   <si>
     <t>waste_liquid_Hom_Salar del Hombre Muerto North</t>
   </si>
   <si>
-    <t>adb46cf1644c4b31a741de20b300074b</t>
+    <t>3c11d67357224d26b72bd407751cca77</t>
   </si>
   <si>
     <t>waste_liquid_Hom</t>
   </si>
   <si>
-    <t>ccde6e4ad4e844b2a655f0d0677afbb3</t>
-  </si>
-  <si>
-    <t>bb835c5690094a0bb23f996a7a13f52c</t>
-  </si>
-  <si>
-    <t>cdd3abdf1e6946e9977bd1be8b84ed59</t>
-  </si>
-  <si>
-    <t>f66d83e3e46743eab35e416bf06f2a67</t>
+    <t>9591ca5f42cb42b7859d4864f384f982</t>
+  </si>
+  <si>
+    <t>62af91237e0b4fa4be0da5a96132346a</t>
+  </si>
+  <si>
+    <t>53bc776915c345368868b277a2b42abd</t>
+  </si>
+  <si>
+    <t>841b6d8f221e4be791bc2707e2331be2</t>
   </si>
   <si>
     <t>waste_liquid_Pas_Salar de Pastos Grandes</t>
   </si>
   <si>
-    <t>4db4c2240c2a4eddab580e390c439a1b</t>
+    <t>1b95231e790741c2a2c343b15f565354</t>
   </si>
   <si>
     <t>waste_liquid_Pas</t>
@@ -3484,46 +3484,46 @@
     <t>waste_liquid_Poz_Pozuelos</t>
   </si>
   <si>
-    <t>7c013ea90c984603913359a5bde04d91</t>
+    <t>6107d30272604525be0054e6f4b5ac3a</t>
   </si>
   <si>
     <t>waste_liquid_Poz</t>
   </si>
   <si>
-    <t>882f404f4b7b4430a6ae0a59fb9246ca</t>
-  </si>
-  <si>
-    <t>4072fab011c54ab2a55955faaea5b89a</t>
+    <t>f6f9683d2c7541188261831daa885b1e</t>
+  </si>
+  <si>
+    <t>c20ca3edd75846bb80c5533db2d9c6d9</t>
   </si>
   <si>
     <t>waste_liquid_Tol_Salar de Tolillar</t>
   </si>
   <si>
-    <t>840492469e8b48d7b221f4c35bd7e332</t>
+    <t>e4cd975ffffd44fd893d1b033e20d4c0</t>
   </si>
   <si>
     <t>waste_liquid_Tol</t>
   </si>
   <si>
-    <t>4e37ce6a0db84fff898e095fc97e6326</t>
-  </si>
-  <si>
-    <t>08b54c7ae5984c2ca0874c50150c4d08</t>
+    <t>269dcae6c3024484a35b419b57d7d25f</t>
+  </si>
+  <si>
+    <t>5f51a3b274db420498b7f8b86008b683</t>
   </si>
   <si>
     <t>waste_liquid_Vid_Sal de Vida</t>
   </si>
   <si>
-    <t>a57b8b55bbf44226a2f3afeeb09b7966</t>
+    <t>a0c62cd3c3914c84ab16b54c74594df1</t>
   </si>
   <si>
     <t>waste_liquid_Vid</t>
   </si>
   <si>
-    <t>b0c2d82df0ad4e25a5e12d2fbe3e05b1</t>
-  </si>
-  <si>
-    <t>e915cccc9e904a82b2f7cc111ee5c955</t>
+    <t>f369bd3969ac4bc8a4d879b5fb8b9162</t>
+  </si>
+  <si>
+    <t>c09a9c402e644838a60605de2abc558c</t>
   </si>
 </sst>
 </file>

</xml_diff>